<commit_message>
Clearer label on the automatic-message switch
</commit_message>
<xml_diff>
--- a/docs/amharic-review.xlsx
+++ b/docs/amharic-review.xlsx
@@ -6796,10 +6796,10 @@
     <t>sms.sendThis</t>
   </si>
   <si>
-    <t>Send this message</t>
-  </si>
-  <si>
-    <t>ይህን መልዕክት ላክ</t>
+    <t>Send this message automatically</t>
+  </si>
+  <si>
+    <t>ይህን መልዕክት በራስ-ሰር ላክ</t>
   </si>
   <si>
     <t>sms.sendTo</t>

</xml_diff>

<commit_message>
SMS schedule and rules: one row per rule with explanation and control
</commit_message>
<xml_diff>
--- a/docs/amharic-review.xlsx
+++ b/docs/amharic-review.xlsx
@@ -6214,6 +6214,15 @@
     <t>0 ገደብ የለም ማለት ነው። ማስታወቂያዎችና ሙከራዎች አይቆጠሩም።</t>
   </si>
   <si>
+    <t>sms.daysBefore</t>
+  </si>
+  <si>
+    <t>days before</t>
+  </si>
+  <si>
+    <t>ቀን በፊት</t>
+  </si>
+  <si>
     <t>sms.daysLate</t>
   </si>
   <si>
@@ -6526,6 +6535,15 @@
     <t>ያለፉ ደረሰኞችን ከዚህ በኋላ አስታውስ</t>
   </si>
   <si>
+    <t>sms.perDay</t>
+  </si>
+  <si>
+    <t>per day</t>
+  </si>
+  <si>
+    <t>በቀን</t>
+  </si>
+  <si>
     <t>sms.ph.amount</t>
   </si>
   <si>
@@ -6719,6 +6737,33 @@
   </si>
   <si>
     <t>ያልተሳኩትን ሁሉ እንደገና ሞክር</t>
+  </si>
+  <si>
+    <t>sms.ruleBeforeTitle</t>
+  </si>
+  <si>
+    <t>Reminder before the due date</t>
+  </si>
+  <si>
+    <t>ከመክፈያ ቀን በፊት ማስታወሻ</t>
+  </si>
+  <si>
+    <t>sms.ruleExtrasTitle</t>
+  </si>
+  <si>
+    <t>Other messages</t>
+  </si>
+  <si>
+    <t>ሌሎች መልዕክቶች</t>
+  </si>
+  <si>
+    <t>sms.ruleQuietTitle</t>
+  </si>
+  <si>
+    <t>Quiet hours</t>
+  </si>
+  <si>
+    <t>የዝምታ ሰዓት</t>
   </si>
   <si>
     <t>sms.rulesApprover</t>
@@ -17878,10 +17923,10 @@
         <v>2126</v>
       </c>
       <c r="C743" t="s">
-        <v>925</v>
+        <v>2127</v>
       </c>
       <c r="D743" t="s">
-        <v>2127</v>
+        <v>2128</v>
       </c>
     </row>
     <row r="744">
@@ -17889,10 +17934,10 @@
         <v>1594</v>
       </c>
       <c r="B744" t="s">
-        <v>2128</v>
+        <v>2129</v>
       </c>
       <c r="C744" t="s">
-        <v>2129</v>
+        <v>925</v>
       </c>
       <c r="D744" t="s">
         <v>2130</v>
@@ -18130,10 +18175,10 @@
         <v>2179</v>
       </c>
       <c r="C761" t="s">
-        <v>306</v>
+        <v>2180</v>
       </c>
       <c r="D761" t="s">
-        <v>307</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="762">
@@ -18141,13 +18186,13 @@
         <v>1594</v>
       </c>
       <c r="B762" t="s">
-        <v>2180</v>
+        <v>2182</v>
       </c>
       <c r="C762" t="s">
-        <v>2181</v>
+        <v>2183</v>
       </c>
       <c r="D762" t="s">
-        <v>2182</v>
+        <v>2184</v>
       </c>
     </row>
     <row r="763">
@@ -18155,13 +18200,13 @@
         <v>1594</v>
       </c>
       <c r="B763" t="s">
-        <v>2183</v>
+        <v>2185</v>
       </c>
       <c r="C763" t="s">
-        <v>2184</v>
+        <v>306</v>
       </c>
       <c r="D763" t="s">
-        <v>2185</v>
+        <v>307</v>
       </c>
     </row>
     <row r="764">
@@ -18200,10 +18245,10 @@
         <v>2192</v>
       </c>
       <c r="C766" t="s">
-        <v>503</v>
+        <v>2193</v>
       </c>
       <c r="D766" t="s">
-        <v>504</v>
+        <v>2194</v>
       </c>
     </row>
     <row r="767">
@@ -18211,13 +18256,13 @@
         <v>1594</v>
       </c>
       <c r="B767" t="s">
-        <v>2193</v>
+        <v>2195</v>
       </c>
       <c r="C767" t="s">
-        <v>2194</v>
+        <v>2196</v>
       </c>
       <c r="D767" t="s">
-        <v>2195</v>
+        <v>2197</v>
       </c>
     </row>
     <row r="768">
@@ -18225,13 +18270,13 @@
         <v>1594</v>
       </c>
       <c r="B768" t="s">
-        <v>2196</v>
+        <v>2198</v>
       </c>
       <c r="C768" t="s">
-        <v>2197</v>
+        <v>503</v>
       </c>
       <c r="D768" t="s">
-        <v>2198</v>
+        <v>504</v>
       </c>
     </row>
     <row r="769">
@@ -18242,10 +18287,10 @@
         <v>2199</v>
       </c>
       <c r="C769" t="s">
-        <v>744</v>
+        <v>2200</v>
       </c>
       <c r="D769" t="s">
-        <v>745</v>
+        <v>2201</v>
       </c>
     </row>
     <row r="770">
@@ -18253,13 +18298,13 @@
         <v>1594</v>
       </c>
       <c r="B770" t="s">
-        <v>2200</v>
+        <v>2202</v>
       </c>
       <c r="C770" t="s">
-        <v>2201</v>
+        <v>2203</v>
       </c>
       <c r="D770" t="s">
-        <v>2202</v>
+        <v>2204</v>
       </c>
     </row>
     <row r="771">
@@ -18267,13 +18312,13 @@
         <v>1594</v>
       </c>
       <c r="B771" t="s">
-        <v>2203</v>
+        <v>2205</v>
       </c>
       <c r="C771" t="s">
-        <v>2204</v>
+        <v>744</v>
       </c>
       <c r="D771" t="s">
-        <v>2205</v>
+        <v>745</v>
       </c>
     </row>
     <row r="772">
@@ -18399,7 +18444,7 @@
         <v>2231</v>
       </c>
       <c r="D780" t="s">
-        <v>733</v>
+        <v>2232</v>
       </c>
     </row>
     <row r="781">
@@ -18407,13 +18452,13 @@
         <v>1594</v>
       </c>
       <c r="B781" t="s">
-        <v>2232</v>
+        <v>2233</v>
       </c>
       <c r="C781" t="s">
-        <v>2233</v>
+        <v>2234</v>
       </c>
       <c r="D781" t="s">
-        <v>2234</v>
+        <v>2235</v>
       </c>
     </row>
     <row r="782">
@@ -18421,13 +18466,13 @@
         <v>1594</v>
       </c>
       <c r="B782" t="s">
-        <v>2235</v>
+        <v>2236</v>
       </c>
       <c r="C782" t="s">
-        <v>2236</v>
+        <v>2237</v>
       </c>
       <c r="D782" t="s">
-        <v>2237</v>
+        <v>733</v>
       </c>
     </row>
     <row r="783">
@@ -18483,7 +18528,7 @@
         <v>2248</v>
       </c>
       <c r="D786" t="s">
-        <v>142</v>
+        <v>2249</v>
       </c>
     </row>
     <row r="787">
@@ -18491,13 +18536,13 @@
         <v>1594</v>
       </c>
       <c r="B787" t="s">
-        <v>2249</v>
+        <v>2250</v>
       </c>
       <c r="C787" t="s">
-        <v>2250</v>
+        <v>2251</v>
       </c>
       <c r="D787" t="s">
-        <v>1557</v>
+        <v>2252</v>
       </c>
     </row>
     <row r="788">
@@ -18505,13 +18550,13 @@
         <v>1594</v>
       </c>
       <c r="B788" t="s">
-        <v>2251</v>
+        <v>2253</v>
       </c>
       <c r="C788" t="s">
-        <v>2252</v>
+        <v>2254</v>
       </c>
       <c r="D788" t="s">
-        <v>1557</v>
+        <v>2255</v>
       </c>
     </row>
     <row r="789">
@@ -18519,13 +18564,13 @@
         <v>1594</v>
       </c>
       <c r="B789" t="s">
-        <v>2253</v>
+        <v>2256</v>
       </c>
       <c r="C789" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="D789" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
     </row>
     <row r="790">
@@ -18533,13 +18578,13 @@
         <v>1594</v>
       </c>
       <c r="B790" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="C790" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="D790" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
     </row>
     <row r="791">
@@ -18547,13 +18592,13 @@
         <v>1594</v>
       </c>
       <c r="B791" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="C791" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="D791" t="s">
-        <v>2261</v>
+        <v>142</v>
       </c>
     </row>
     <row r="792">
@@ -18561,13 +18606,13 @@
         <v>1594</v>
       </c>
       <c r="B792" t="s">
-        <v>2262</v>
+        <v>2264</v>
       </c>
       <c r="C792" t="s">
-        <v>2263</v>
+        <v>2265</v>
       </c>
       <c r="D792" t="s">
-        <v>2264</v>
+        <v>1557</v>
       </c>
     </row>
     <row r="793">
@@ -18575,13 +18620,13 @@
         <v>1594</v>
       </c>
       <c r="B793" t="s">
-        <v>2265</v>
+        <v>2266</v>
       </c>
       <c r="C793" t="s">
-        <v>2266</v>
+        <v>2267</v>
       </c>
       <c r="D793" t="s">
-        <v>2267</v>
+        <v>1557</v>
       </c>
     </row>
     <row r="794">
@@ -18732,10 +18777,10 @@
         <v>2298</v>
       </c>
       <c r="C804" t="s">
-        <v>2106</v>
+        <v>2299</v>
       </c>
       <c r="D804" t="s">
-        <v>2107</v>
+        <v>2300</v>
       </c>
     </row>
     <row r="805">
@@ -18743,13 +18788,13 @@
         <v>1594</v>
       </c>
       <c r="B805" t="s">
-        <v>2299</v>
+        <v>2301</v>
       </c>
       <c r="C805" t="s">
-        <v>2300</v>
+        <v>2302</v>
       </c>
       <c r="D805" t="s">
-        <v>2301</v>
+        <v>2303</v>
       </c>
     </row>
     <row r="806">
@@ -18757,13 +18802,13 @@
         <v>1594</v>
       </c>
       <c r="B806" t="s">
-        <v>2302</v>
+        <v>2304</v>
       </c>
       <c r="C806" t="s">
-        <v>2115</v>
+        <v>2305</v>
       </c>
       <c r="D806" t="s">
-        <v>2116</v>
+        <v>2306</v>
       </c>
     </row>
     <row r="807">
@@ -18771,13 +18816,13 @@
         <v>1594</v>
       </c>
       <c r="B807" t="s">
-        <v>2303</v>
+        <v>2307</v>
       </c>
       <c r="C807" t="s">
-        <v>2304</v>
+        <v>2308</v>
       </c>
       <c r="D807" t="s">
-        <v>2305</v>
+        <v>2309</v>
       </c>
     </row>
     <row r="808">
@@ -18785,13 +18830,13 @@
         <v>1594</v>
       </c>
       <c r="B808" t="s">
-        <v>2306</v>
+        <v>2310</v>
       </c>
       <c r="C808" t="s">
-        <v>2118</v>
+        <v>2311</v>
       </c>
       <c r="D808" t="s">
-        <v>2119</v>
+        <v>2312</v>
       </c>
     </row>
     <row r="809">
@@ -18799,13 +18844,13 @@
         <v>1594</v>
       </c>
       <c r="B809" t="s">
-        <v>2307</v>
+        <v>2313</v>
       </c>
       <c r="C809" t="s">
-        <v>2308</v>
+        <v>2109</v>
       </c>
       <c r="D809" t="s">
-        <v>2309</v>
+        <v>2110</v>
       </c>
     </row>
     <row r="810">
@@ -18813,13 +18858,13 @@
         <v>1594</v>
       </c>
       <c r="B810" t="s">
-        <v>2310</v>
+        <v>2314</v>
       </c>
       <c r="C810" t="s">
-        <v>2311</v>
+        <v>2315</v>
       </c>
       <c r="D810" t="s">
-        <v>2312</v>
+        <v>2316</v>
       </c>
     </row>
     <row r="811">
@@ -18827,13 +18872,13 @@
         <v>1594</v>
       </c>
       <c r="B811" t="s">
-        <v>2313</v>
+        <v>2317</v>
       </c>
       <c r="C811" t="s">
-        <v>2314</v>
+        <v>2118</v>
       </c>
       <c r="D811" t="s">
-        <v>2315</v>
+        <v>2119</v>
       </c>
     </row>
     <row r="812">
@@ -18841,13 +18886,13 @@
         <v>1594</v>
       </c>
       <c r="B812" t="s">
-        <v>2316</v>
+        <v>2318</v>
       </c>
       <c r="C812" t="s">
-        <v>2317</v>
+        <v>2319</v>
       </c>
       <c r="D812" t="s">
-        <v>2318</v>
+        <v>2320</v>
       </c>
     </row>
     <row r="813">
@@ -18855,13 +18900,13 @@
         <v>1594</v>
       </c>
       <c r="B813" t="s">
-        <v>2319</v>
+        <v>2321</v>
       </c>
       <c r="C813" t="s">
-        <v>2320</v>
+        <v>2121</v>
       </c>
       <c r="D813" t="s">
-        <v>2321</v>
+        <v>2122</v>
       </c>
     </row>
     <row r="814">
@@ -18886,10 +18931,10 @@
         <v>2325</v>
       </c>
       <c r="C815" t="s">
-        <v>1904</v>
+        <v>2326</v>
       </c>
       <c r="D815" t="s">
-        <v>444</v>
+        <v>2327</v>
       </c>
     </row>
     <row r="816">
@@ -18897,13 +18942,13 @@
         <v>1594</v>
       </c>
       <c r="B816" t="s">
-        <v>2326</v>
+        <v>2328</v>
       </c>
       <c r="C816" t="s">
-        <v>2327</v>
+        <v>2329</v>
       </c>
       <c r="D816" t="s">
-        <v>2328</v>
+        <v>2330</v>
       </c>
     </row>
     <row r="817">
@@ -18911,13 +18956,13 @@
         <v>1594</v>
       </c>
       <c r="B817" t="s">
-        <v>2329</v>
+        <v>2331</v>
       </c>
       <c r="C817" t="s">
-        <v>2330</v>
+        <v>2332</v>
       </c>
       <c r="D817" t="s">
-        <v>2331</v>
+        <v>2333</v>
       </c>
     </row>
     <row r="818">
@@ -18925,102 +18970,102 @@
         <v>1594</v>
       </c>
       <c r="B818" t="s">
-        <v>2332</v>
+        <v>2334</v>
       </c>
       <c r="C818" t="s">
-        <v>2333</v>
+        <v>2335</v>
       </c>
       <c r="D818" t="s">
-        <v>2334</v>
+        <v>2336</v>
       </c>
     </row>
     <row r="819">
       <c r="A819" t="s">
-        <v>1609</v>
+        <v>1594</v>
       </c>
       <c r="B819" t="s">
-        <v>2335</v>
+        <v>2337</v>
       </c>
       <c r="C819" t="s">
-        <v>832</v>
+        <v>2338</v>
       </c>
       <c r="D819" t="s">
-        <v>833</v>
+        <v>2339</v>
       </c>
     </row>
     <row r="820">
       <c r="A820" t="s">
-        <v>1609</v>
+        <v>1594</v>
       </c>
       <c r="B820" t="s">
-        <v>2336</v>
+        <v>2340</v>
       </c>
       <c r="C820" t="s">
-        <v>2337</v>
+        <v>1904</v>
       </c>
       <c r="D820" t="s">
-        <v>2338</v>
+        <v>444</v>
       </c>
     </row>
     <row r="821">
       <c r="A821" t="s">
-        <v>1609</v>
+        <v>1594</v>
       </c>
       <c r="B821" t="s">
-        <v>2339</v>
+        <v>2341</v>
       </c>
       <c r="C821" t="s">
-        <v>2340</v>
+        <v>2342</v>
       </c>
       <c r="D821" t="s">
-        <v>2341</v>
+        <v>2343</v>
       </c>
     </row>
     <row r="822">
       <c r="A822" t="s">
-        <v>2342</v>
+        <v>1594</v>
       </c>
       <c r="B822" t="s">
-        <v>2343</v>
+        <v>2344</v>
       </c>
       <c r="C822" t="s">
-        <v>2342</v>
+        <v>2345</v>
       </c>
       <c r="D822" t="s">
-        <v>2344</v>
+        <v>2346</v>
       </c>
     </row>
     <row r="823">
       <c r="A823" t="s">
-        <v>2342</v>
+        <v>1594</v>
       </c>
       <c r="B823" t="s">
-        <v>2345</v>
+        <v>2347</v>
       </c>
       <c r="C823" t="s">
-        <v>2346</v>
+        <v>2348</v>
       </c>
       <c r="D823" t="s">
-        <v>2347</v>
+        <v>2349</v>
       </c>
     </row>
     <row r="824">
       <c r="A824" t="s">
-        <v>2342</v>
+        <v>1609</v>
       </c>
       <c r="B824" t="s">
-        <v>2348</v>
+        <v>2350</v>
       </c>
       <c r="C824" t="s">
-        <v>2349</v>
+        <v>832</v>
       </c>
       <c r="D824" t="s">
-        <v>2350</v>
+        <v>833</v>
       </c>
     </row>
     <row r="825">
       <c r="A825" t="s">
-        <v>2342</v>
+        <v>1609</v>
       </c>
       <c r="B825" t="s">
         <v>2351</v>
@@ -19034,7 +19079,7 @@
     </row>
     <row r="826">
       <c r="A826" t="s">
-        <v>1612</v>
+        <v>1609</v>
       </c>
       <c r="B826" t="s">
         <v>2354</v>
@@ -19048,13 +19093,13 @@
     </row>
     <row r="827">
       <c r="A827" t="s">
-        <v>1612</v>
+        <v>2357</v>
       </c>
       <c r="B827" t="s">
+        <v>2358</v>
+      </c>
+      <c r="C827" t="s">
         <v>2357</v>
-      </c>
-      <c r="C827" t="s">
-        <v>2358</v>
       </c>
       <c r="D827" t="s">
         <v>2359</v>
@@ -19062,7 +19107,7 @@
     </row>
     <row r="828">
       <c r="A828" t="s">
-        <v>1612</v>
+        <v>2357</v>
       </c>
       <c r="B828" t="s">
         <v>2360</v>
@@ -19076,30 +19121,30 @@
     </row>
     <row r="829">
       <c r="A829" t="s">
-        <v>1612</v>
+        <v>2357</v>
       </c>
       <c r="B829" t="s">
         <v>2363</v>
       </c>
       <c r="C829" t="s">
-        <v>280</v>
+        <v>2364</v>
       </c>
       <c r="D829" t="s">
-        <v>281</v>
+        <v>2365</v>
       </c>
     </row>
     <row r="830">
       <c r="A830" t="s">
-        <v>1612</v>
+        <v>2357</v>
       </c>
       <c r="B830" t="s">
-        <v>2364</v>
+        <v>2366</v>
       </c>
       <c r="C830" t="s">
-        <v>2365</v>
+        <v>2367</v>
       </c>
       <c r="D830" t="s">
-        <v>1764</v>
+        <v>2368</v>
       </c>
     </row>
     <row r="831">
@@ -19107,13 +19152,13 @@
         <v>1612</v>
       </c>
       <c r="B831" t="s">
-        <v>2366</v>
+        <v>2369</v>
       </c>
       <c r="C831" t="s">
-        <v>2367</v>
+        <v>2370</v>
       </c>
       <c r="D831" t="s">
-        <v>2368</v>
+        <v>2371</v>
       </c>
     </row>
     <row r="832">
@@ -19121,13 +19166,13 @@
         <v>1612</v>
       </c>
       <c r="B832" t="s">
-        <v>2369</v>
+        <v>2372</v>
       </c>
       <c r="C832" t="s">
-        <v>2370</v>
+        <v>2373</v>
       </c>
       <c r="D832" t="s">
-        <v>2371</v>
+        <v>2374</v>
       </c>
     </row>
     <row r="833">
@@ -19135,13 +19180,13 @@
         <v>1612</v>
       </c>
       <c r="B833" t="s">
-        <v>2372</v>
+        <v>2375</v>
       </c>
       <c r="C833" t="s">
-        <v>2373</v>
+        <v>2376</v>
       </c>
       <c r="D833" t="s">
-        <v>2374</v>
+        <v>2377</v>
       </c>
     </row>
     <row r="834">
@@ -19149,13 +19194,13 @@
         <v>1612</v>
       </c>
       <c r="B834" t="s">
-        <v>2375</v>
+        <v>2378</v>
       </c>
       <c r="C834" t="s">
-        <v>2376</v>
+        <v>280</v>
       </c>
       <c r="D834" t="s">
-        <v>2377</v>
+        <v>281</v>
       </c>
     </row>
     <row r="835">
@@ -19163,13 +19208,13 @@
         <v>1612</v>
       </c>
       <c r="B835" t="s">
-        <v>2378</v>
+        <v>2379</v>
       </c>
       <c r="C835" t="s">
-        <v>2379</v>
+        <v>2380</v>
       </c>
       <c r="D835" t="s">
-        <v>2380</v>
+        <v>1764</v>
       </c>
     </row>
     <row r="836">
@@ -19278,10 +19323,10 @@
         <v>2402</v>
       </c>
       <c r="C843" t="s">
-        <v>2376</v>
+        <v>2403</v>
       </c>
       <c r="D843" t="s">
-        <v>2377</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="844">
@@ -19289,13 +19334,13 @@
         <v>1612</v>
       </c>
       <c r="B844" t="s">
-        <v>2403</v>
+        <v>2405</v>
       </c>
       <c r="C844" t="s">
-        <v>2404</v>
+        <v>2406</v>
       </c>
       <c r="D844" t="s">
-        <v>2405</v>
+        <v>2407</v>
       </c>
     </row>
     <row r="845">
@@ -19303,13 +19348,13 @@
         <v>1612</v>
       </c>
       <c r="B845" t="s">
-        <v>2406</v>
+        <v>2408</v>
       </c>
       <c r="C845" t="s">
-        <v>2407</v>
+        <v>2409</v>
       </c>
       <c r="D845" t="s">
-        <v>2408</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="846">
@@ -19317,13 +19362,13 @@
         <v>1612</v>
       </c>
       <c r="B846" t="s">
-        <v>2409</v>
+        <v>2411</v>
       </c>
       <c r="C846" t="s">
-        <v>2410</v>
+        <v>2412</v>
       </c>
       <c r="D846" t="s">
-        <v>2411</v>
+        <v>2413</v>
       </c>
     </row>
     <row r="847">
@@ -19331,13 +19376,13 @@
         <v>1612</v>
       </c>
       <c r="B847" t="s">
-        <v>2412</v>
+        <v>2414</v>
       </c>
       <c r="C847" t="s">
-        <v>2413</v>
+        <v>2415</v>
       </c>
       <c r="D847" t="s">
-        <v>2414</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="848">
@@ -19345,13 +19390,13 @@
         <v>1612</v>
       </c>
       <c r="B848" t="s">
-        <v>2415</v>
+        <v>2417</v>
       </c>
       <c r="C848" t="s">
-        <v>2416</v>
+        <v>2391</v>
       </c>
       <c r="D848" t="s">
-        <v>2417</v>
+        <v>2392</v>
       </c>
     </row>
     <row r="849">
@@ -19404,10 +19449,10 @@
         <v>2427</v>
       </c>
       <c r="C852" t="s">
-        <v>2367</v>
+        <v>2428</v>
       </c>
       <c r="D852" t="s">
-        <v>2368</v>
+        <v>2429</v>
       </c>
     </row>
     <row r="853">
@@ -19415,13 +19460,13 @@
         <v>1612</v>
       </c>
       <c r="B853" t="s">
-        <v>2428</v>
+        <v>2430</v>
       </c>
       <c r="C853" t="s">
-        <v>2429</v>
+        <v>2431</v>
       </c>
       <c r="D853" t="s">
-        <v>2430</v>
+        <v>2432</v>
       </c>
     </row>
     <row r="854">
@@ -19429,13 +19474,13 @@
         <v>1612</v>
       </c>
       <c r="B854" t="s">
-        <v>2431</v>
+        <v>2433</v>
       </c>
       <c r="C854" t="s">
-        <v>2432</v>
+        <v>2434</v>
       </c>
       <c r="D854" t="s">
-        <v>2433</v>
+        <v>2435</v>
       </c>
     </row>
     <row r="855">
@@ -19443,13 +19488,13 @@
         <v>1612</v>
       </c>
       <c r="B855" t="s">
-        <v>2434</v>
+        <v>2436</v>
       </c>
       <c r="C855" t="s">
-        <v>2435</v>
+        <v>2437</v>
       </c>
       <c r="D855" t="s">
-        <v>2436</v>
+        <v>2438</v>
       </c>
     </row>
     <row r="856">
@@ -19457,13 +19502,13 @@
         <v>1612</v>
       </c>
       <c r="B856" t="s">
-        <v>2437</v>
+        <v>2439</v>
       </c>
       <c r="C856" t="s">
-        <v>2438</v>
+        <v>2440</v>
       </c>
       <c r="D856" t="s">
-        <v>2439</v>
+        <v>2441</v>
       </c>
     </row>
     <row r="857">
@@ -19471,13 +19516,13 @@
         <v>1612</v>
       </c>
       <c r="B857" t="s">
-        <v>2440</v>
+        <v>2442</v>
       </c>
       <c r="C857" t="s">
-        <v>2441</v>
+        <v>2382</v>
       </c>
       <c r="D857" t="s">
-        <v>2442</v>
+        <v>2383</v>
       </c>
     </row>
     <row r="858">
@@ -19544,10 +19589,10 @@
         <v>2455</v>
       </c>
       <c r="C862" t="s">
-        <v>1240</v>
+        <v>2456</v>
       </c>
       <c r="D862" t="s">
-        <v>1241</v>
+        <v>2457</v>
       </c>
     </row>
     <row r="863">
@@ -19555,13 +19600,13 @@
         <v>1612</v>
       </c>
       <c r="B863" t="s">
-        <v>2456</v>
+        <v>2458</v>
       </c>
       <c r="C863" t="s">
-        <v>2457</v>
+        <v>2459</v>
       </c>
       <c r="D863" t="s">
-        <v>2458</v>
+        <v>2460</v>
       </c>
     </row>
     <row r="864">
@@ -19569,13 +19614,13 @@
         <v>1612</v>
       </c>
       <c r="B864" t="s">
-        <v>2459</v>
+        <v>2461</v>
       </c>
       <c r="C864" t="s">
-        <v>2460</v>
+        <v>2462</v>
       </c>
       <c r="D864" t="s">
-        <v>2461</v>
+        <v>2463</v>
       </c>
     </row>
     <row r="865">
@@ -19583,13 +19628,13 @@
         <v>1612</v>
       </c>
       <c r="B865" t="s">
-        <v>2462</v>
+        <v>2464</v>
       </c>
       <c r="C865" t="s">
-        <v>2463</v>
+        <v>2465</v>
       </c>
       <c r="D865" t="s">
-        <v>2464</v>
+        <v>2466</v>
       </c>
     </row>
     <row r="866">
@@ -19597,13 +19642,83 @@
         <v>1612</v>
       </c>
       <c r="B866" t="s">
-        <v>2465</v>
+        <v>2467</v>
       </c>
       <c r="C866" t="s">
-        <v>2466</v>
+        <v>2468</v>
       </c>
       <c r="D866" t="s">
-        <v>2467</v>
+        <v>2469</v>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B867" t="s">
+        <v>2470</v>
+      </c>
+      <c r="C867" t="s">
+        <v>1240</v>
+      </c>
+      <c r="D867" t="s">
+        <v>1241</v>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B868" t="s">
+        <v>2471</v>
+      </c>
+      <c r="C868" t="s">
+        <v>2472</v>
+      </c>
+      <c r="D868" t="s">
+        <v>2473</v>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B869" t="s">
+        <v>2474</v>
+      </c>
+      <c r="C869" t="s">
+        <v>2475</v>
+      </c>
+      <c r="D869" t="s">
+        <v>2476</v>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B870" t="s">
+        <v>2477</v>
+      </c>
+      <c r="C870" t="s">
+        <v>2478</v>
+      </c>
+      <c r="D870" t="s">
+        <v>2479</v>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B871" t="s">
+        <v>2480</v>
+      </c>
+      <c r="C871" t="s">
+        <v>2481</v>
+      </c>
+      <c r="D871" t="s">
+        <v>2482</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Reports: key figures and charts above every report
</commit_message>
<xml_diff>
--- a/docs/amharic-review.xlsx
+++ b/docs/amharic-review.xlsx
@@ -5830,6 +5830,132 @@
     <t>የውዝፍ ዕዳ ዕድሜ</t>
   </si>
   <si>
+    <t>rep.c.ageing</t>
+  </si>
+  <si>
+    <t>Where the arrears sit</t>
+  </si>
+  <si>
+    <t>ውዝፍ የት እንዳለ</t>
+  </si>
+  <si>
+    <t>rep.c.balanceOverTime</t>
+  </si>
+  <si>
+    <t>Balance over time</t>
+  </si>
+  <si>
+    <t>ቀሪ ሂሳብ በጊዜ ሂደት</t>
+  </si>
+  <si>
+    <t>rep.c.biggestDeposits</t>
+  </si>
+  <si>
+    <t>Largest deposits held</t>
+  </si>
+  <si>
+    <t>ትልቁ ተይዞ ያለ ዋስትና</t>
+  </si>
+  <si>
+    <t>rep.c.biggestRent</t>
+  </si>
+  <si>
+    <t>Rent by lease</t>
+  </si>
+  <si>
+    <t>ኪራይ በውል</t>
+  </si>
+  <si>
+    <t>rep.c.depositMix</t>
+  </si>
+  <si>
+    <t>Where the deposits stand</t>
+  </si>
+  <si>
+    <t>የዋስትና ሁኔታ</t>
+  </si>
+  <si>
+    <t>rep.c.endingByMonth</t>
+  </si>
+  <si>
+    <t>Rent of leases ending, by month</t>
+  </si>
+  <si>
+    <t>የሚያበቁ ውሎች ኪራይ በወር</t>
+  </si>
+  <si>
+    <t>rep.c.occupancy</t>
+  </si>
+  <si>
+    <t>የክፍል አጠቃቀም</t>
+  </si>
+  <si>
+    <t>rep.c.rate</t>
+  </si>
+  <si>
+    <t>Collection rate by month</t>
+  </si>
+  <si>
+    <t>የስብሰባ መጠን በወር</t>
+  </si>
+  <si>
+    <t>rep.c.rentByBuilding</t>
+  </si>
+  <si>
+    <t>Rent by building</t>
+  </si>
+  <si>
+    <t>ኪራይ በሕንፃ</t>
+  </si>
+  <si>
+    <t>rep.c.rentByCategory</t>
+  </si>
+  <si>
+    <t>Rent by category</t>
+  </si>
+  <si>
+    <t>ኪራይ በምድብ</t>
+  </si>
+  <si>
+    <t>rep.c.topDebtors</t>
+  </si>
+  <si>
+    <t>Largest balances</t>
+  </si>
+  <si>
+    <t>ትልቁ ቀሪ ሂሳብ</t>
+  </si>
+  <si>
+    <t>rep.c.trend</t>
+  </si>
+  <si>
+    <t>Billed and collected</t>
+  </si>
+  <si>
+    <t>የወጣና የተሰበሰበ</t>
+  </si>
+  <si>
+    <t>rep.c.vacantArea</t>
+  </si>
+  <si>
+    <t>Vacant area by category</t>
+  </si>
+  <si>
+    <t>ክፍት ስፋት በምድብ</t>
+  </si>
+  <si>
+    <t>rep.c.vacantByCategory</t>
+  </si>
+  <si>
+    <t>Rent waiting to be let, by category</t>
+  </si>
+  <si>
+    <t>ለመከራየት የሚጠብቅ ኪራይ በምድብ</t>
+  </si>
+  <si>
+    <t>rep.collected</t>
+  </si>
+  <si>
     <t>rep.collectedNote</t>
   </si>
   <si>
@@ -5875,6 +6001,276 @@
     <t>የውል ማብቂያ</t>
   </si>
   <si>
+    <t>rep.k.bestMonth</t>
+  </si>
+  <si>
+    <t>Best month collected</t>
+  </si>
+  <si>
+    <t>ብዙ የተሰበሰበበት ወር</t>
+  </si>
+  <si>
+    <t>rep.k.charged</t>
+  </si>
+  <si>
+    <t>Charged</t>
+  </si>
+  <si>
+    <t>የተጠየቀ</t>
+  </si>
+  <si>
+    <t>rep.k.covered</t>
+  </si>
+  <si>
+    <t>covered</t>
+  </si>
+  <si>
+    <t>የተሸፈነ</t>
+  </si>
+  <si>
+    <t>rep.k.entries</t>
+  </si>
+  <si>
+    <t>entries</t>
+  </si>
+  <si>
+    <t>መዝገቦች</t>
+  </si>
+  <si>
+    <t>rep.k.largest</t>
+  </si>
+  <si>
+    <t>Largest balance</t>
+  </si>
+  <si>
+    <t>rep.k.let</t>
+  </si>
+  <si>
+    <t>let</t>
+  </si>
+  <si>
+    <t>የተከራየ</t>
+  </si>
+  <si>
+    <t>rep.k.monthlyRent</t>
+  </si>
+  <si>
+    <t>Monthly rent</t>
+  </si>
+  <si>
+    <t>ወርሃዊ ኪራይ</t>
+  </si>
+  <si>
+    <t>rep.k.months</t>
+  </si>
+  <si>
+    <t>months</t>
+  </si>
+  <si>
+    <t>ወራት</t>
+  </si>
+  <si>
+    <t>rep.k.needsAction</t>
+  </si>
+  <si>
+    <t>Renew or close them</t>
+  </si>
+  <si>
+    <t>ያድሱ ወይም ይዝጉ</t>
+  </si>
+  <si>
+    <t>rep.k.none</t>
+  </si>
+  <si>
+    <t>ምንም</t>
+  </si>
+  <si>
+    <t>rep.k.notLet</t>
+  </si>
+  <si>
+    <t>not let</t>
+  </si>
+  <si>
+    <t>ያልተከራየ</t>
+  </si>
+  <si>
+    <t>rep.k.ofBilled</t>
+  </si>
+  <si>
+    <t>ከወጣው</t>
+  </si>
+  <si>
+    <t>rep.k.ofCharged</t>
+  </si>
+  <si>
+    <t>of charged</t>
+  </si>
+  <si>
+    <t>ከተጠየቀው</t>
+  </si>
+  <si>
+    <t>rep.k.ofOutstanding</t>
+  </si>
+  <si>
+    <t>of outstanding</t>
+  </si>
+  <si>
+    <t>ከቀሪው</t>
+  </si>
+  <si>
+    <t>rep.k.ofUnits</t>
+  </si>
+  <si>
+    <t>of all units</t>
+  </si>
+  <si>
+    <t>ከሁሉም ክፍሎች</t>
+  </si>
+  <si>
+    <t>rep.k.other</t>
+  </si>
+  <si>
+    <t>Reserved or in repair</t>
+  </si>
+  <si>
+    <t>የተያዙ ወይም በጥገና</t>
+  </si>
+  <si>
+    <t>rep.k.otherNote</t>
+  </si>
+  <si>
+    <t>not available to let</t>
+  </si>
+  <si>
+    <t>ለመከራየት የማይገኙ</t>
+  </si>
+  <si>
+    <t>rep.k.over90</t>
+  </si>
+  <si>
+    <t>Over 90 days</t>
+  </si>
+  <si>
+    <t>ከ90 ቀን በላይ</t>
+  </si>
+  <si>
+    <t>rep.k.overdue</t>
+  </si>
+  <si>
+    <t>ያለፈ</t>
+  </si>
+  <si>
+    <t>rep.k.paid</t>
+  </si>
+  <si>
+    <t>rep.k.pastEnd</t>
+  </si>
+  <si>
+    <t>Past end</t>
+  </si>
+  <si>
+    <t>rep.k.potential</t>
+  </si>
+  <si>
+    <t>Rent waiting to be let</t>
+  </si>
+  <si>
+    <t>ለመከራየት የሚጠብቅ ኪራይ</t>
+  </si>
+  <si>
+    <t>rep.k.received</t>
+  </si>
+  <si>
+    <t>received</t>
+  </si>
+  <si>
+    <t>የደረሰ</t>
+  </si>
+  <si>
+    <t>rep.k.refundsDue</t>
+  </si>
+  <si>
+    <t>refunds due</t>
+  </si>
+  <si>
+    <t>የሚመለሱ</t>
+  </si>
+  <si>
+    <t>rep.k.renters</t>
+  </si>
+  <si>
+    <t>renters owing</t>
+  </si>
+  <si>
+    <t>ተከራዮች ዕዳ ያለባቸው</t>
+  </si>
+  <si>
+    <t>rep.k.rentPerM2</t>
+  </si>
+  <si>
+    <t>Average rent per m²</t>
+  </si>
+  <si>
+    <t>አማካይ ኪራይ በካሬ ሜትር</t>
+  </si>
+  <si>
+    <t>rep.k.required</t>
+  </si>
+  <si>
+    <t>Deposits required</t>
+  </si>
+  <si>
+    <t>የሚያስፈልግ ዋስትና</t>
+  </si>
+  <si>
+    <t>rep.k.settled</t>
+  </si>
+  <si>
+    <t>Settled</t>
+  </si>
+  <si>
+    <t>rep.k.shortfallNote</t>
+  </si>
+  <si>
+    <t>held below what leases require</t>
+  </si>
+  <si>
+    <t>ከውሎች መስፈርት በታች ተይዞ ያለ</t>
+  </si>
+  <si>
+    <t>rep.k.units</t>
+  </si>
+  <si>
+    <t>units</t>
+  </si>
+  <si>
+    <t>rep.k.vacantArea</t>
+  </si>
+  <si>
+    <t>Vacant area</t>
+  </si>
+  <si>
+    <t>ክፍት ስፋት</t>
+  </si>
+  <si>
+    <t>rep.k.vacantUnits</t>
+  </si>
+  <si>
+    <t>Vacant units</t>
+  </si>
+  <si>
+    <t>ክፍት ክፍሎች</t>
+  </si>
+  <si>
+    <t>rep.k.yearly</t>
+  </si>
+  <si>
+    <t>per year</t>
+  </si>
+  <si>
+    <t>በዓመት</t>
+  </si>
+  <si>
     <t>rep.leases</t>
   </si>
   <si>
@@ -5905,6 +6301,15 @@
     <t>ከማብቂያ ቀናቸው ያለፉና ገና ያልተዘጉ</t>
   </si>
   <si>
+    <t>rep.pastEndTitle</t>
+  </si>
+  <si>
+    <t>Past their end date</t>
+  </si>
+  <si>
+    <t>ማብቂያ ቀናቸው ያለፈ</t>
+  </si>
+  <si>
     <t>rep.refundDue</t>
   </si>
   <si>
@@ -6404,9 +6809,6 @@
   </si>
   <si>
     <t>sms.kpi.delivered</t>
-  </si>
-  <si>
-    <t>የደረሰ</t>
   </si>
   <si>
     <t>sms.kpi.queued</t>
@@ -17100,7 +17502,7 @@
         <v>1954</v>
       </c>
       <c r="D684" t="s">
-        <v>1352</v>
+        <v>1955</v>
       </c>
     </row>
     <row r="685">
@@ -17108,10 +17510,10 @@
         <v>1603</v>
       </c>
       <c r="B685" t="s">
-        <v>1955</v>
+        <v>1956</v>
       </c>
       <c r="C685" t="s">
-        <v>1956</v>
+        <v>1685</v>
       </c>
       <c r="D685" t="s">
         <v>1957</v>
@@ -17125,10 +17527,10 @@
         <v>1958</v>
       </c>
       <c r="C686" t="s">
-        <v>1614</v>
+        <v>1959</v>
       </c>
       <c r="D686" t="s">
-        <v>1629</v>
+        <v>1960</v>
       </c>
     </row>
     <row r="687">
@@ -17136,13 +17538,13 @@
         <v>1603</v>
       </c>
       <c r="B687" t="s">
-        <v>1959</v>
+        <v>1961</v>
       </c>
       <c r="C687" t="s">
-        <v>42</v>
+        <v>1962</v>
       </c>
       <c r="D687" t="s">
-        <v>43</v>
+        <v>1963</v>
       </c>
     </row>
     <row r="688">
@@ -17150,13 +17552,13 @@
         <v>1603</v>
       </c>
       <c r="B688" t="s">
-        <v>1960</v>
+        <v>1964</v>
       </c>
       <c r="C688" t="s">
-        <v>1961</v>
+        <v>1965</v>
       </c>
       <c r="D688" t="s">
-        <v>1962</v>
+        <v>1966</v>
       </c>
     </row>
     <row r="689">
@@ -17164,13 +17566,13 @@
         <v>1603</v>
       </c>
       <c r="B689" t="s">
-        <v>1963</v>
+        <v>1967</v>
       </c>
       <c r="C689" t="s">
-        <v>1964</v>
+        <v>1968</v>
       </c>
       <c r="D689" t="s">
-        <v>1965</v>
+        <v>1969</v>
       </c>
     </row>
     <row r="690">
@@ -17178,13 +17580,13 @@
         <v>1603</v>
       </c>
       <c r="B690" t="s">
-        <v>1966</v>
+        <v>1970</v>
       </c>
       <c r="C690" t="s">
-        <v>1967</v>
+        <v>1971</v>
       </c>
       <c r="D690" t="s">
-        <v>1968</v>
+        <v>1972</v>
       </c>
     </row>
     <row r="691">
@@ -17192,13 +17594,13 @@
         <v>1603</v>
       </c>
       <c r="B691" t="s">
-        <v>1969</v>
+        <v>1973</v>
       </c>
       <c r="C691" t="s">
-        <v>1970</v>
+        <v>1974</v>
       </c>
       <c r="D691" t="s">
-        <v>1971</v>
+        <v>1975</v>
       </c>
     </row>
     <row r="692">
@@ -17206,13 +17608,13 @@
         <v>1603</v>
       </c>
       <c r="B692" t="s">
-        <v>1972</v>
+        <v>1976</v>
       </c>
       <c r="C692" t="s">
-        <v>1973</v>
+        <v>1977</v>
       </c>
       <c r="D692" t="s">
-        <v>1974</v>
+        <v>1978</v>
       </c>
     </row>
     <row r="693">
@@ -17220,13 +17622,13 @@
         <v>1603</v>
       </c>
       <c r="B693" t="s">
-        <v>1975</v>
+        <v>1979</v>
       </c>
       <c r="C693" t="s">
-        <v>1976</v>
+        <v>346</v>
       </c>
       <c r="D693" t="s">
-        <v>1977</v>
+        <v>347</v>
       </c>
     </row>
     <row r="694">
@@ -17234,13 +17636,13 @@
         <v>1603</v>
       </c>
       <c r="B694" t="s">
-        <v>1978</v>
+        <v>1980</v>
       </c>
       <c r="C694" t="s">
-        <v>1979</v>
+        <v>1981</v>
       </c>
       <c r="D694" t="s">
-        <v>1980</v>
+        <v>1982</v>
       </c>
     </row>
     <row r="695">
@@ -17248,13 +17650,13 @@
         <v>1603</v>
       </c>
       <c r="B695" t="s">
-        <v>1981</v>
+        <v>1983</v>
       </c>
       <c r="C695" t="s">
-        <v>1982</v>
+        <v>1984</v>
       </c>
       <c r="D695" t="s">
-        <v>1983</v>
+        <v>1985</v>
       </c>
     </row>
     <row r="696">
@@ -17262,13 +17664,13 @@
         <v>1603</v>
       </c>
       <c r="B696" t="s">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="C696" t="s">
-        <v>1985</v>
+        <v>1987</v>
       </c>
       <c r="D696" t="s">
-        <v>1986</v>
+        <v>1988</v>
       </c>
     </row>
     <row r="697">
@@ -17276,13 +17678,13 @@
         <v>1603</v>
       </c>
       <c r="B697" t="s">
-        <v>1987</v>
+        <v>1989</v>
       </c>
       <c r="C697" t="s">
-        <v>1988</v>
+        <v>1990</v>
       </c>
       <c r="D697" t="s">
-        <v>1989</v>
+        <v>1991</v>
       </c>
     </row>
     <row r="698">
@@ -17290,13 +17692,13 @@
         <v>1603</v>
       </c>
       <c r="B698" t="s">
-        <v>1990</v>
+        <v>1992</v>
       </c>
       <c r="C698" t="s">
-        <v>1991</v>
+        <v>1993</v>
       </c>
       <c r="D698" t="s">
-        <v>1992</v>
+        <v>1994</v>
       </c>
     </row>
     <row r="699">
@@ -17304,74 +17706,74 @@
         <v>1603</v>
       </c>
       <c r="B699" t="s">
-        <v>1993</v>
+        <v>1995</v>
       </c>
       <c r="C699" t="s">
-        <v>1994</v>
+        <v>1996</v>
       </c>
       <c r="D699" t="s">
-        <v>1995</v>
+        <v>1997</v>
       </c>
     </row>
     <row r="700">
       <c r="A700" t="s">
-        <v>1996</v>
+        <v>1603</v>
       </c>
       <c r="B700" t="s">
-        <v>1997</v>
+        <v>1998</v>
       </c>
       <c r="C700" t="s">
-        <v>1998</v>
+        <v>1999</v>
       </c>
       <c r="D700" t="s">
-        <v>1999</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="701">
       <c r="A701" t="s">
-        <v>1996</v>
+        <v>1603</v>
       </c>
       <c r="B701" t="s">
-        <v>2000</v>
+        <v>2001</v>
       </c>
       <c r="C701" t="s">
-        <v>2001</v>
+        <v>2002</v>
       </c>
       <c r="D701" t="s">
-        <v>2002</v>
+        <v>2003</v>
       </c>
     </row>
     <row r="702">
       <c r="A702" t="s">
-        <v>1996</v>
+        <v>1603</v>
       </c>
       <c r="B702" t="s">
-        <v>2003</v>
+        <v>2004</v>
       </c>
       <c r="C702" t="s">
-        <v>2004</v>
+        <v>2005</v>
       </c>
       <c r="D702" t="s">
-        <v>2005</v>
+        <v>2006</v>
       </c>
     </row>
     <row r="703">
       <c r="A703" t="s">
-        <v>1996</v>
+        <v>1603</v>
       </c>
       <c r="B703" t="s">
-        <v>2006</v>
+        <v>2007</v>
       </c>
       <c r="C703" t="s">
-        <v>2007</v>
+        <v>2008</v>
       </c>
       <c r="D703" t="s">
-        <v>2008</v>
+        <v>1969</v>
       </c>
     </row>
     <row r="704">
       <c r="A704" t="s">
-        <v>1278</v>
+        <v>1603</v>
       </c>
       <c r="B704" t="s">
         <v>2009</v>
@@ -17385,7 +17787,7 @@
     </row>
     <row r="705">
       <c r="A705" t="s">
-        <v>1278</v>
+        <v>1603</v>
       </c>
       <c r="B705" t="s">
         <v>2012</v>
@@ -17399,7 +17801,7 @@
     </row>
     <row r="706">
       <c r="A706" t="s">
-        <v>1278</v>
+        <v>1603</v>
       </c>
       <c r="B706" t="s">
         <v>2015</v>
@@ -17413,7 +17815,7 @@
     </row>
     <row r="707">
       <c r="A707" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B707" t="s">
         <v>2018</v>
@@ -17427,674 +17829,674 @@
     </row>
     <row r="708">
       <c r="A708" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B708" t="s">
         <v>2021</v>
       </c>
       <c r="C708" t="s">
+        <v>1166</v>
+      </c>
+      <c r="D708" t="s">
         <v>2022</v>
-      </c>
-      <c r="D708" t="s">
-        <v>2023</v>
       </c>
     </row>
     <row r="709">
       <c r="A709" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B709" t="s">
+        <v>2023</v>
+      </c>
+      <c r="C709" t="s">
         <v>2024</v>
       </c>
-      <c r="C709" t="s">
+      <c r="D709" t="s">
         <v>2025</v>
-      </c>
-      <c r="D709" t="s">
-        <v>2026</v>
       </c>
     </row>
     <row r="710">
       <c r="A710" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B710" t="s">
+        <v>2026</v>
+      </c>
+      <c r="C710" t="s">
+        <v>357</v>
+      </c>
+      <c r="D710" t="s">
         <v>2027</v>
-      </c>
-      <c r="C710" t="s">
-        <v>2028</v>
-      </c>
-      <c r="D710" t="s">
-        <v>2029</v>
       </c>
     </row>
     <row r="711">
       <c r="A711" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B711" t="s">
+        <v>2028</v>
+      </c>
+      <c r="C711" t="s">
+        <v>2029</v>
+      </c>
+      <c r="D711" t="s">
         <v>2030</v>
-      </c>
-      <c r="C711" t="s">
-        <v>2031</v>
-      </c>
-      <c r="D711" t="s">
-        <v>2032</v>
       </c>
     </row>
     <row r="712">
       <c r="A712" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B712" t="s">
+        <v>2031</v>
+      </c>
+      <c r="C712" t="s">
+        <v>2032</v>
+      </c>
+      <c r="D712" t="s">
         <v>2033</v>
-      </c>
-      <c r="C712" t="s">
-        <v>2034</v>
-      </c>
-      <c r="D712" t="s">
-        <v>2035</v>
       </c>
     </row>
     <row r="713">
       <c r="A713" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B713" t="s">
+        <v>2034</v>
+      </c>
+      <c r="C713" t="s">
+        <v>2035</v>
+      </c>
+      <c r="D713" t="s">
         <v>2036</v>
-      </c>
-      <c r="C713" t="s">
-        <v>2037</v>
-      </c>
-      <c r="D713" t="s">
-        <v>2038</v>
       </c>
     </row>
     <row r="714">
       <c r="A714" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B714" t="s">
+        <v>2037</v>
+      </c>
+      <c r="C714" t="s">
+        <v>2038</v>
+      </c>
+      <c r="D714" t="s">
         <v>2039</v>
-      </c>
-      <c r="C714" t="s">
-        <v>2040</v>
-      </c>
-      <c r="D714" t="s">
-        <v>2041</v>
       </c>
     </row>
     <row r="715">
       <c r="A715" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B715" t="s">
+        <v>2040</v>
+      </c>
+      <c r="C715" t="s">
+        <v>2041</v>
+      </c>
+      <c r="D715" t="s">
         <v>2042</v>
-      </c>
-      <c r="C715" t="s">
-        <v>2043</v>
-      </c>
-      <c r="D715" t="s">
-        <v>2044</v>
       </c>
     </row>
     <row r="716">
       <c r="A716" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B716" t="s">
+        <v>2043</v>
+      </c>
+      <c r="C716" t="s">
+        <v>2044</v>
+      </c>
+      <c r="D716" t="s">
         <v>2045</v>
-      </c>
-      <c r="C716" t="s">
-        <v>2046</v>
-      </c>
-      <c r="D716" t="s">
-        <v>2047</v>
       </c>
     </row>
     <row r="717">
       <c r="A717" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B717" t="s">
-        <v>2048</v>
+        <v>2046</v>
       </c>
       <c r="C717" t="s">
-        <v>2049</v>
+        <v>352</v>
       </c>
       <c r="D717" t="s">
-        <v>2050</v>
+        <v>2047</v>
       </c>
     </row>
     <row r="718">
       <c r="A718" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B718" t="s">
-        <v>2051</v>
+        <v>2048</v>
       </c>
       <c r="C718" t="s">
-        <v>2052</v>
+        <v>369</v>
       </c>
       <c r="D718" t="s">
-        <v>2053</v>
+        <v>370</v>
       </c>
     </row>
     <row r="719">
       <c r="A719" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B719" t="s">
-        <v>2054</v>
+        <v>2049</v>
       </c>
       <c r="C719" t="s">
-        <v>2055</v>
+        <v>2050</v>
       </c>
       <c r="D719" t="s">
-        <v>2056</v>
+        <v>2047</v>
       </c>
     </row>
     <row r="720">
       <c r="A720" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B720" t="s">
-        <v>2057</v>
+        <v>2051</v>
       </c>
       <c r="C720" t="s">
-        <v>2058</v>
+        <v>2052</v>
       </c>
       <c r="D720" t="s">
-        <v>2059</v>
+        <v>2053</v>
       </c>
     </row>
     <row r="721">
       <c r="A721" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B721" t="s">
-        <v>2060</v>
+        <v>2054</v>
       </c>
       <c r="C721" t="s">
-        <v>2061</v>
+        <v>2055</v>
       </c>
       <c r="D721" t="s">
-        <v>2062</v>
+        <v>2056</v>
       </c>
     </row>
     <row r="722">
       <c r="A722" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B722" t="s">
-        <v>2063</v>
+        <v>2057</v>
       </c>
       <c r="C722" t="s">
-        <v>2064</v>
+        <v>2058</v>
       </c>
       <c r="D722" t="s">
-        <v>2065</v>
+        <v>2059</v>
       </c>
     </row>
     <row r="723">
       <c r="A723" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B723" t="s">
-        <v>2066</v>
+        <v>2060</v>
       </c>
       <c r="C723" t="s">
-        <v>2067</v>
+        <v>2061</v>
       </c>
       <c r="D723" t="s">
-        <v>2068</v>
+        <v>2062</v>
       </c>
     </row>
     <row r="724">
       <c r="A724" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B724" t="s">
-        <v>2069</v>
+        <v>2063</v>
       </c>
       <c r="C724" t="s">
-        <v>2070</v>
+        <v>2064</v>
       </c>
       <c r="D724" t="s">
-        <v>2071</v>
+        <v>2065</v>
       </c>
     </row>
     <row r="725">
       <c r="A725" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B725" t="s">
-        <v>2072</v>
+        <v>2066</v>
       </c>
       <c r="C725" t="s">
-        <v>2073</v>
+        <v>2067</v>
       </c>
       <c r="D725" t="s">
-        <v>2074</v>
+        <v>2068</v>
       </c>
     </row>
     <row r="726">
       <c r="A726" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B726" t="s">
-        <v>2075</v>
+        <v>2069</v>
       </c>
       <c r="C726" t="s">
-        <v>2076</v>
+        <v>2070</v>
       </c>
       <c r="D726" t="s">
-        <v>2077</v>
+        <v>2003</v>
       </c>
     </row>
     <row r="727">
       <c r="A727" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B727" t="s">
-        <v>2078</v>
+        <v>2071</v>
       </c>
       <c r="C727" t="s">
-        <v>2079</v>
+        <v>2072</v>
       </c>
       <c r="D727" t="s">
-        <v>2080</v>
+        <v>2073</v>
       </c>
     </row>
     <row r="728">
       <c r="A728" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B728" t="s">
-        <v>2081</v>
+        <v>2074</v>
       </c>
       <c r="C728" t="s">
-        <v>2082</v>
+        <v>2075</v>
       </c>
       <c r="D728" t="s">
-        <v>2083</v>
+        <v>1557</v>
       </c>
     </row>
     <row r="729">
       <c r="A729" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B729" t="s">
-        <v>2084</v>
+        <v>2076</v>
       </c>
       <c r="C729" t="s">
-        <v>2085</v>
+        <v>2077</v>
       </c>
       <c r="D729" t="s">
-        <v>2086</v>
+        <v>2078</v>
       </c>
     </row>
     <row r="730">
       <c r="A730" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B730" t="s">
-        <v>2087</v>
+        <v>2079</v>
       </c>
       <c r="C730" t="s">
-        <v>2088</v>
+        <v>2080</v>
       </c>
       <c r="D730" t="s">
-        <v>2089</v>
+        <v>2081</v>
       </c>
     </row>
     <row r="731">
       <c r="A731" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B731" t="s">
-        <v>2090</v>
+        <v>2082</v>
       </c>
       <c r="C731" t="s">
-        <v>2091</v>
+        <v>2083</v>
       </c>
       <c r="D731" t="s">
-        <v>2092</v>
+        <v>2084</v>
       </c>
     </row>
     <row r="732">
       <c r="A732" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B732" t="s">
-        <v>2093</v>
+        <v>2085</v>
       </c>
       <c r="C732" t="s">
-        <v>2094</v>
+        <v>2086</v>
       </c>
       <c r="D732" t="s">
-        <v>2095</v>
+        <v>1352</v>
       </c>
     </row>
     <row r="733">
       <c r="A733" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B733" t="s">
-        <v>2096</v>
+        <v>2087</v>
       </c>
       <c r="C733" t="s">
-        <v>2097</v>
+        <v>2088</v>
       </c>
       <c r="D733" t="s">
-        <v>2098</v>
+        <v>2089</v>
       </c>
     </row>
     <row r="734">
       <c r="A734" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B734" t="s">
-        <v>2099</v>
+        <v>2090</v>
       </c>
       <c r="C734" t="s">
-        <v>2100</v>
+        <v>1614</v>
       </c>
       <c r="D734" t="s">
-        <v>2101</v>
+        <v>1629</v>
       </c>
     </row>
     <row r="735">
       <c r="A735" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B735" t="s">
-        <v>2102</v>
+        <v>2091</v>
       </c>
       <c r="C735" t="s">
-        <v>2103</v>
+        <v>42</v>
       </c>
       <c r="D735" t="s">
-        <v>2104</v>
+        <v>43</v>
       </c>
     </row>
     <row r="736">
       <c r="A736" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B736" t="s">
-        <v>2105</v>
+        <v>2092</v>
       </c>
       <c r="C736" t="s">
-        <v>2106</v>
+        <v>2093</v>
       </c>
       <c r="D736" t="s">
-        <v>2107</v>
+        <v>2094</v>
       </c>
     </row>
     <row r="737">
       <c r="A737" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B737" t="s">
-        <v>2108</v>
+        <v>2095</v>
       </c>
       <c r="C737" t="s">
-        <v>2109</v>
+        <v>2096</v>
       </c>
       <c r="D737" t="s">
-        <v>2110</v>
+        <v>2097</v>
       </c>
     </row>
     <row r="738">
       <c r="A738" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B738" t="s">
-        <v>2111</v>
+        <v>2098</v>
       </c>
       <c r="C738" t="s">
-        <v>2112</v>
+        <v>2099</v>
       </c>
       <c r="D738" t="s">
-        <v>2113</v>
+        <v>2100</v>
       </c>
     </row>
     <row r="739">
       <c r="A739" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B739" t="s">
-        <v>2114</v>
+        <v>2101</v>
       </c>
       <c r="C739" t="s">
-        <v>2115</v>
+        <v>2102</v>
       </c>
       <c r="D739" t="s">
-        <v>2116</v>
+        <v>2103</v>
       </c>
     </row>
     <row r="740">
       <c r="A740" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B740" t="s">
-        <v>2117</v>
+        <v>2104</v>
       </c>
       <c r="C740" t="s">
-        <v>2118</v>
+        <v>2105</v>
       </c>
       <c r="D740" t="s">
-        <v>2119</v>
+        <v>2106</v>
       </c>
     </row>
     <row r="741">
       <c r="A741" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B741" t="s">
-        <v>2120</v>
+        <v>2107</v>
       </c>
       <c r="C741" t="s">
-        <v>2121</v>
+        <v>2108</v>
       </c>
       <c r="D741" t="s">
-        <v>2122</v>
+        <v>2109</v>
       </c>
     </row>
     <row r="742">
       <c r="A742" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B742" t="s">
-        <v>2123</v>
+        <v>2110</v>
       </c>
       <c r="C742" t="s">
-        <v>2124</v>
+        <v>2111</v>
       </c>
       <c r="D742" t="s">
-        <v>2125</v>
+        <v>2112</v>
       </c>
     </row>
     <row r="743">
       <c r="A743" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B743" t="s">
-        <v>2126</v>
+        <v>2113</v>
       </c>
       <c r="C743" t="s">
-        <v>2127</v>
+        <v>2114</v>
       </c>
       <c r="D743" t="s">
-        <v>2128</v>
+        <v>2115</v>
       </c>
     </row>
     <row r="744">
       <c r="A744" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B744" t="s">
-        <v>2129</v>
+        <v>2116</v>
       </c>
       <c r="C744" t="s">
-        <v>925</v>
+        <v>2117</v>
       </c>
       <c r="D744" t="s">
-        <v>2130</v>
+        <v>2118</v>
       </c>
     </row>
     <row r="745">
       <c r="A745" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B745" t="s">
-        <v>2131</v>
+        <v>2119</v>
       </c>
       <c r="C745" t="s">
-        <v>2132</v>
+        <v>2120</v>
       </c>
       <c r="D745" t="s">
-        <v>2133</v>
+        <v>2121</v>
       </c>
     </row>
     <row r="746">
       <c r="A746" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B746" t="s">
-        <v>2134</v>
+        <v>2122</v>
       </c>
       <c r="C746" t="s">
-        <v>2135</v>
+        <v>2123</v>
       </c>
       <c r="D746" t="s">
-        <v>2136</v>
+        <v>2124</v>
       </c>
     </row>
     <row r="747">
       <c r="A747" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B747" t="s">
-        <v>2137</v>
+        <v>2125</v>
       </c>
       <c r="C747" t="s">
-        <v>2138</v>
+        <v>2126</v>
       </c>
       <c r="D747" t="s">
-        <v>2139</v>
+        <v>2127</v>
       </c>
     </row>
     <row r="748">
       <c r="A748" t="s">
-        <v>1594</v>
+        <v>1603</v>
       </c>
       <c r="B748" t="s">
-        <v>2140</v>
+        <v>2128</v>
       </c>
       <c r="C748" t="s">
-        <v>2141</v>
+        <v>2129</v>
       </c>
       <c r="D748" t="s">
-        <v>2142</v>
+        <v>2130</v>
       </c>
     </row>
     <row r="749">
       <c r="A749" t="s">
-        <v>1594</v>
+        <v>2131</v>
       </c>
       <c r="B749" t="s">
-        <v>2143</v>
+        <v>2132</v>
       </c>
       <c r="C749" t="s">
-        <v>2144</v>
+        <v>2133</v>
       </c>
       <c r="D749" t="s">
-        <v>2145</v>
+        <v>2134</v>
       </c>
     </row>
     <row r="750">
       <c r="A750" t="s">
-        <v>1594</v>
+        <v>2131</v>
       </c>
       <c r="B750" t="s">
-        <v>2146</v>
+        <v>2135</v>
       </c>
       <c r="C750" t="s">
-        <v>2147</v>
+        <v>2136</v>
       </c>
       <c r="D750" t="s">
-        <v>2148</v>
+        <v>2137</v>
       </c>
     </row>
     <row r="751">
       <c r="A751" t="s">
-        <v>1594</v>
+        <v>2131</v>
       </c>
       <c r="B751" t="s">
-        <v>2149</v>
+        <v>2138</v>
       </c>
       <c r="C751" t="s">
-        <v>2150</v>
+        <v>2139</v>
       </c>
       <c r="D751" t="s">
-        <v>2151</v>
+        <v>2140</v>
       </c>
     </row>
     <row r="752">
       <c r="A752" t="s">
-        <v>1594</v>
+        <v>2131</v>
       </c>
       <c r="B752" t="s">
-        <v>2152</v>
+        <v>2141</v>
       </c>
       <c r="C752" t="s">
-        <v>2153</v>
+        <v>2142</v>
       </c>
       <c r="D752" t="s">
-        <v>2154</v>
+        <v>2143</v>
       </c>
     </row>
     <row r="753">
       <c r="A753" t="s">
-        <v>1594</v>
+        <v>1278</v>
       </c>
       <c r="B753" t="s">
-        <v>2155</v>
+        <v>2144</v>
       </c>
       <c r="C753" t="s">
-        <v>2156</v>
+        <v>2145</v>
       </c>
       <c r="D753" t="s">
-        <v>2157</v>
+        <v>2146</v>
       </c>
     </row>
     <row r="754">
       <c r="A754" t="s">
-        <v>1594</v>
+        <v>1278</v>
       </c>
       <c r="B754" t="s">
-        <v>2158</v>
+        <v>2147</v>
       </c>
       <c r="C754" t="s">
-        <v>2159</v>
+        <v>2148</v>
       </c>
       <c r="D754" t="s">
-        <v>2160</v>
+        <v>2149</v>
       </c>
     </row>
     <row r="755">
       <c r="A755" t="s">
-        <v>1594</v>
+        <v>1278</v>
       </c>
       <c r="B755" t="s">
-        <v>2161</v>
+        <v>2150</v>
       </c>
       <c r="C755" t="s">
-        <v>2162</v>
+        <v>2151</v>
       </c>
       <c r="D755" t="s">
-        <v>2163</v>
+        <v>2152</v>
       </c>
     </row>
     <row r="756">
@@ -18102,13 +18504,13 @@
         <v>1594</v>
       </c>
       <c r="B756" t="s">
-        <v>2164</v>
+        <v>2153</v>
       </c>
       <c r="C756" t="s">
-        <v>2165</v>
+        <v>2154</v>
       </c>
       <c r="D756" t="s">
-        <v>2166</v>
+        <v>2155</v>
       </c>
     </row>
     <row r="757">
@@ -18116,13 +18518,13 @@
         <v>1594</v>
       </c>
       <c r="B757" t="s">
-        <v>2167</v>
+        <v>2156</v>
       </c>
       <c r="C757" t="s">
-        <v>2168</v>
+        <v>2157</v>
       </c>
       <c r="D757" t="s">
-        <v>2169</v>
+        <v>2158</v>
       </c>
     </row>
     <row r="758">
@@ -18130,13 +18532,13 @@
         <v>1594</v>
       </c>
       <c r="B758" t="s">
-        <v>2170</v>
+        <v>2159</v>
       </c>
       <c r="C758" t="s">
-        <v>2171</v>
+        <v>2160</v>
       </c>
       <c r="D758" t="s">
-        <v>2172</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="759">
@@ -18144,13 +18546,13 @@
         <v>1594</v>
       </c>
       <c r="B759" t="s">
-        <v>2173</v>
+        <v>2162</v>
       </c>
       <c r="C759" t="s">
-        <v>2174</v>
+        <v>2163</v>
       </c>
       <c r="D759" t="s">
-        <v>2175</v>
+        <v>2164</v>
       </c>
     </row>
     <row r="760">
@@ -18158,13 +18560,13 @@
         <v>1594</v>
       </c>
       <c r="B760" t="s">
-        <v>2176</v>
+        <v>2165</v>
       </c>
       <c r="C760" t="s">
-        <v>2177</v>
+        <v>2166</v>
       </c>
       <c r="D760" t="s">
-        <v>2178</v>
+        <v>2167</v>
       </c>
     </row>
     <row r="761">
@@ -18172,13 +18574,13 @@
         <v>1594</v>
       </c>
       <c r="B761" t="s">
-        <v>2179</v>
+        <v>2168</v>
       </c>
       <c r="C761" t="s">
-        <v>2180</v>
+        <v>2169</v>
       </c>
       <c r="D761" t="s">
-        <v>2181</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="762">
@@ -18186,13 +18588,13 @@
         <v>1594</v>
       </c>
       <c r="B762" t="s">
-        <v>2182</v>
+        <v>2171</v>
       </c>
       <c r="C762" t="s">
-        <v>2183</v>
+        <v>2172</v>
       </c>
       <c r="D762" t="s">
-        <v>2184</v>
+        <v>2173</v>
       </c>
     </row>
     <row r="763">
@@ -18200,13 +18602,13 @@
         <v>1594</v>
       </c>
       <c r="B763" t="s">
-        <v>2185</v>
+        <v>2174</v>
       </c>
       <c r="C763" t="s">
-        <v>306</v>
+        <v>2175</v>
       </c>
       <c r="D763" t="s">
-        <v>307</v>
+        <v>2176</v>
       </c>
     </row>
     <row r="764">
@@ -18214,13 +18616,13 @@
         <v>1594</v>
       </c>
       <c r="B764" t="s">
-        <v>2186</v>
+        <v>2177</v>
       </c>
       <c r="C764" t="s">
-        <v>2187</v>
+        <v>2178</v>
       </c>
       <c r="D764" t="s">
-        <v>2188</v>
+        <v>2179</v>
       </c>
     </row>
     <row r="765">
@@ -18228,13 +18630,13 @@
         <v>1594</v>
       </c>
       <c r="B765" t="s">
-        <v>2189</v>
+        <v>2180</v>
       </c>
       <c r="C765" t="s">
-        <v>2190</v>
+        <v>2181</v>
       </c>
       <c r="D765" t="s">
-        <v>2191</v>
+        <v>2182</v>
       </c>
     </row>
     <row r="766">
@@ -18242,13 +18644,13 @@
         <v>1594</v>
       </c>
       <c r="B766" t="s">
-        <v>2192</v>
+        <v>2183</v>
       </c>
       <c r="C766" t="s">
-        <v>2193</v>
+        <v>2184</v>
       </c>
       <c r="D766" t="s">
-        <v>2194</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="767">
@@ -18256,13 +18658,13 @@
         <v>1594</v>
       </c>
       <c r="B767" t="s">
-        <v>2195</v>
+        <v>2186</v>
       </c>
       <c r="C767" t="s">
-        <v>2196</v>
+        <v>2187</v>
       </c>
       <c r="D767" t="s">
-        <v>2197</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="768">
@@ -18270,13 +18672,13 @@
         <v>1594</v>
       </c>
       <c r="B768" t="s">
-        <v>2198</v>
+        <v>2189</v>
       </c>
       <c r="C768" t="s">
-        <v>503</v>
+        <v>2190</v>
       </c>
       <c r="D768" t="s">
-        <v>504</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="769">
@@ -18284,13 +18686,13 @@
         <v>1594</v>
       </c>
       <c r="B769" t="s">
-        <v>2199</v>
+        <v>2192</v>
       </c>
       <c r="C769" t="s">
-        <v>2200</v>
+        <v>2193</v>
       </c>
       <c r="D769" t="s">
-        <v>2201</v>
+        <v>2194</v>
       </c>
     </row>
     <row r="770">
@@ -18298,13 +18700,13 @@
         <v>1594</v>
       </c>
       <c r="B770" t="s">
-        <v>2202</v>
+        <v>2195</v>
       </c>
       <c r="C770" t="s">
-        <v>2203</v>
+        <v>2196</v>
       </c>
       <c r="D770" t="s">
-        <v>2204</v>
+        <v>2197</v>
       </c>
     </row>
     <row r="771">
@@ -18312,13 +18714,13 @@
         <v>1594</v>
       </c>
       <c r="B771" t="s">
-        <v>2205</v>
+        <v>2198</v>
       </c>
       <c r="C771" t="s">
-        <v>744</v>
+        <v>2199</v>
       </c>
       <c r="D771" t="s">
-        <v>745</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="772">
@@ -18326,13 +18728,13 @@
         <v>1594</v>
       </c>
       <c r="B772" t="s">
-        <v>2206</v>
+        <v>2201</v>
       </c>
       <c r="C772" t="s">
-        <v>2207</v>
+        <v>2202</v>
       </c>
       <c r="D772" t="s">
-        <v>2208</v>
+        <v>2203</v>
       </c>
     </row>
     <row r="773">
@@ -18340,13 +18742,13 @@
         <v>1594</v>
       </c>
       <c r="B773" t="s">
-        <v>2209</v>
+        <v>2204</v>
       </c>
       <c r="C773" t="s">
-        <v>2210</v>
+        <v>2205</v>
       </c>
       <c r="D773" t="s">
-        <v>2211</v>
+        <v>2206</v>
       </c>
     </row>
     <row r="774">
@@ -18354,13 +18756,13 @@
         <v>1594</v>
       </c>
       <c r="B774" t="s">
-        <v>2212</v>
+        <v>2207</v>
       </c>
       <c r="C774" t="s">
-        <v>2213</v>
+        <v>2208</v>
       </c>
       <c r="D774" t="s">
-        <v>2214</v>
+        <v>2209</v>
       </c>
     </row>
     <row r="775">
@@ -18368,13 +18770,13 @@
         <v>1594</v>
       </c>
       <c r="B775" t="s">
-        <v>2215</v>
+        <v>2210</v>
       </c>
       <c r="C775" t="s">
-        <v>2216</v>
+        <v>2211</v>
       </c>
       <c r="D775" t="s">
-        <v>2217</v>
+        <v>2212</v>
       </c>
     </row>
     <row r="776">
@@ -18382,13 +18784,13 @@
         <v>1594</v>
       </c>
       <c r="B776" t="s">
-        <v>2218</v>
+        <v>2213</v>
       </c>
       <c r="C776" t="s">
-        <v>2219</v>
+        <v>2214</v>
       </c>
       <c r="D776" t="s">
-        <v>2220</v>
+        <v>2215</v>
       </c>
     </row>
     <row r="777">
@@ -18396,13 +18798,13 @@
         <v>1594</v>
       </c>
       <c r="B777" t="s">
-        <v>2221</v>
+        <v>2216</v>
       </c>
       <c r="C777" t="s">
-        <v>2222</v>
+        <v>2217</v>
       </c>
       <c r="D777" t="s">
-        <v>2223</v>
+        <v>2218</v>
       </c>
     </row>
     <row r="778">
@@ -18410,13 +18812,13 @@
         <v>1594</v>
       </c>
       <c r="B778" t="s">
-        <v>2224</v>
+        <v>2219</v>
       </c>
       <c r="C778" t="s">
-        <v>2225</v>
+        <v>2220</v>
       </c>
       <c r="D778" t="s">
-        <v>2226</v>
+        <v>2221</v>
       </c>
     </row>
     <row r="779">
@@ -18424,13 +18826,13 @@
         <v>1594</v>
       </c>
       <c r="B779" t="s">
-        <v>2227</v>
+        <v>2222</v>
       </c>
       <c r="C779" t="s">
-        <v>2228</v>
+        <v>2223</v>
       </c>
       <c r="D779" t="s">
-        <v>2229</v>
+        <v>2224</v>
       </c>
     </row>
     <row r="780">
@@ -18438,13 +18840,13 @@
         <v>1594</v>
       </c>
       <c r="B780" t="s">
-        <v>2230</v>
+        <v>2225</v>
       </c>
       <c r="C780" t="s">
-        <v>2231</v>
+        <v>2226</v>
       </c>
       <c r="D780" t="s">
-        <v>2232</v>
+        <v>2227</v>
       </c>
     </row>
     <row r="781">
@@ -18452,13 +18854,13 @@
         <v>1594</v>
       </c>
       <c r="B781" t="s">
-        <v>2233</v>
+        <v>2228</v>
       </c>
       <c r="C781" t="s">
-        <v>2234</v>
+        <v>2229</v>
       </c>
       <c r="D781" t="s">
-        <v>2235</v>
+        <v>2230</v>
       </c>
     </row>
     <row r="782">
@@ -18466,13 +18868,13 @@
         <v>1594</v>
       </c>
       <c r="B782" t="s">
-        <v>2236</v>
+        <v>2231</v>
       </c>
       <c r="C782" t="s">
-        <v>2237</v>
+        <v>2232</v>
       </c>
       <c r="D782" t="s">
-        <v>733</v>
+        <v>2233</v>
       </c>
     </row>
     <row r="783">
@@ -18480,13 +18882,13 @@
         <v>1594</v>
       </c>
       <c r="B783" t="s">
-        <v>2238</v>
+        <v>2234</v>
       </c>
       <c r="C783" t="s">
-        <v>2239</v>
+        <v>2235</v>
       </c>
       <c r="D783" t="s">
-        <v>2240</v>
+        <v>2236</v>
       </c>
     </row>
     <row r="784">
@@ -18494,13 +18896,13 @@
         <v>1594</v>
       </c>
       <c r="B784" t="s">
-        <v>2241</v>
+        <v>2237</v>
       </c>
       <c r="C784" t="s">
-        <v>2242</v>
+        <v>2238</v>
       </c>
       <c r="D784" t="s">
-        <v>2243</v>
+        <v>2239</v>
       </c>
     </row>
     <row r="785">
@@ -18508,13 +18910,13 @@
         <v>1594</v>
       </c>
       <c r="B785" t="s">
-        <v>2244</v>
+        <v>2240</v>
       </c>
       <c r="C785" t="s">
-        <v>2245</v>
+        <v>2241</v>
       </c>
       <c r="D785" t="s">
-        <v>2246</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="786">
@@ -18522,13 +18924,13 @@
         <v>1594</v>
       </c>
       <c r="B786" t="s">
-        <v>2247</v>
+        <v>2243</v>
       </c>
       <c r="C786" t="s">
-        <v>2248</v>
+        <v>2244</v>
       </c>
       <c r="D786" t="s">
-        <v>2249</v>
+        <v>2245</v>
       </c>
     </row>
     <row r="787">
@@ -18536,13 +18938,13 @@
         <v>1594</v>
       </c>
       <c r="B787" t="s">
-        <v>2250</v>
+        <v>2246</v>
       </c>
       <c r="C787" t="s">
-        <v>2251</v>
+        <v>2247</v>
       </c>
       <c r="D787" t="s">
-        <v>2252</v>
+        <v>2248</v>
       </c>
     </row>
     <row r="788">
@@ -18550,13 +18952,13 @@
         <v>1594</v>
       </c>
       <c r="B788" t="s">
-        <v>2253</v>
+        <v>2249</v>
       </c>
       <c r="C788" t="s">
-        <v>2254</v>
+        <v>2250</v>
       </c>
       <c r="D788" t="s">
-        <v>2255</v>
+        <v>2251</v>
       </c>
     </row>
     <row r="789">
@@ -18564,13 +18966,13 @@
         <v>1594</v>
       </c>
       <c r="B789" t="s">
-        <v>2256</v>
+        <v>2252</v>
       </c>
       <c r="C789" t="s">
-        <v>2257</v>
+        <v>2253</v>
       </c>
       <c r="D789" t="s">
-        <v>2258</v>
+        <v>2254</v>
       </c>
     </row>
     <row r="790">
@@ -18578,13 +18980,13 @@
         <v>1594</v>
       </c>
       <c r="B790" t="s">
-        <v>2259</v>
+        <v>2255</v>
       </c>
       <c r="C790" t="s">
-        <v>2260</v>
+        <v>2256</v>
       </c>
       <c r="D790" t="s">
-        <v>2261</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="791">
@@ -18592,13 +18994,13 @@
         <v>1594</v>
       </c>
       <c r="B791" t="s">
-        <v>2262</v>
+        <v>2258</v>
       </c>
       <c r="C791" t="s">
-        <v>2263</v>
+        <v>2259</v>
       </c>
       <c r="D791" t="s">
-        <v>142</v>
+        <v>2260</v>
       </c>
     </row>
     <row r="792">
@@ -18606,13 +19008,13 @@
         <v>1594</v>
       </c>
       <c r="B792" t="s">
-        <v>2264</v>
+        <v>2261</v>
       </c>
       <c r="C792" t="s">
-        <v>2265</v>
+        <v>2262</v>
       </c>
       <c r="D792" t="s">
-        <v>1557</v>
+        <v>2263</v>
       </c>
     </row>
     <row r="793">
@@ -18620,13 +19022,13 @@
         <v>1594</v>
       </c>
       <c r="B793" t="s">
-        <v>2266</v>
+        <v>2264</v>
       </c>
       <c r="C793" t="s">
-        <v>2267</v>
+        <v>925</v>
       </c>
       <c r="D793" t="s">
-        <v>1557</v>
+        <v>2056</v>
       </c>
     </row>
     <row r="794">
@@ -18634,13 +19036,13 @@
         <v>1594</v>
       </c>
       <c r="B794" t="s">
-        <v>2268</v>
+        <v>2265</v>
       </c>
       <c r="C794" t="s">
-        <v>2269</v>
+        <v>2266</v>
       </c>
       <c r="D794" t="s">
-        <v>2270</v>
+        <v>2267</v>
       </c>
     </row>
     <row r="795">
@@ -18648,13 +19050,13 @@
         <v>1594</v>
       </c>
       <c r="B795" t="s">
-        <v>2271</v>
+        <v>2268</v>
       </c>
       <c r="C795" t="s">
-        <v>2272</v>
+        <v>2269</v>
       </c>
       <c r="D795" t="s">
-        <v>2273</v>
+        <v>2270</v>
       </c>
     </row>
     <row r="796">
@@ -18662,13 +19064,13 @@
         <v>1594</v>
       </c>
       <c r="B796" t="s">
-        <v>2274</v>
+        <v>2271</v>
       </c>
       <c r="C796" t="s">
-        <v>2275</v>
+        <v>2272</v>
       </c>
       <c r="D796" t="s">
-        <v>2276</v>
+        <v>2273</v>
       </c>
     </row>
     <row r="797">
@@ -18676,13 +19078,13 @@
         <v>1594</v>
       </c>
       <c r="B797" t="s">
-        <v>2277</v>
+        <v>2274</v>
       </c>
       <c r="C797" t="s">
-        <v>2278</v>
+        <v>2275</v>
       </c>
       <c r="D797" t="s">
-        <v>2279</v>
+        <v>2276</v>
       </c>
     </row>
     <row r="798">
@@ -18690,13 +19092,13 @@
         <v>1594</v>
       </c>
       <c r="B798" t="s">
-        <v>2280</v>
+        <v>2277</v>
       </c>
       <c r="C798" t="s">
-        <v>2281</v>
+        <v>2278</v>
       </c>
       <c r="D798" t="s">
-        <v>2282</v>
+        <v>2279</v>
       </c>
     </row>
     <row r="799">
@@ -18704,13 +19106,13 @@
         <v>1594</v>
       </c>
       <c r="B799" t="s">
-        <v>2283</v>
+        <v>2280</v>
       </c>
       <c r="C799" t="s">
-        <v>2284</v>
+        <v>2281</v>
       </c>
       <c r="D799" t="s">
-        <v>2285</v>
+        <v>2282</v>
       </c>
     </row>
     <row r="800">
@@ -18718,13 +19120,13 @@
         <v>1594</v>
       </c>
       <c r="B800" t="s">
-        <v>2286</v>
+        <v>2283</v>
       </c>
       <c r="C800" t="s">
-        <v>2287</v>
+        <v>2284</v>
       </c>
       <c r="D800" t="s">
-        <v>2288</v>
+        <v>2285</v>
       </c>
     </row>
     <row r="801">
@@ -18732,13 +19134,13 @@
         <v>1594</v>
       </c>
       <c r="B801" t="s">
-        <v>2289</v>
+        <v>2286</v>
       </c>
       <c r="C801" t="s">
-        <v>2290</v>
+        <v>2287</v>
       </c>
       <c r="D801" t="s">
-        <v>2291</v>
+        <v>2288</v>
       </c>
     </row>
     <row r="802">
@@ -18746,13 +19148,13 @@
         <v>1594</v>
       </c>
       <c r="B802" t="s">
-        <v>2292</v>
+        <v>2289</v>
       </c>
       <c r="C802" t="s">
-        <v>2293</v>
+        <v>2290</v>
       </c>
       <c r="D802" t="s">
-        <v>2294</v>
+        <v>2291</v>
       </c>
     </row>
     <row r="803">
@@ -18760,13 +19162,13 @@
         <v>1594</v>
       </c>
       <c r="B803" t="s">
-        <v>2295</v>
+        <v>2292</v>
       </c>
       <c r="C803" t="s">
-        <v>2296</v>
+        <v>2293</v>
       </c>
       <c r="D803" t="s">
-        <v>2297</v>
+        <v>2294</v>
       </c>
     </row>
     <row r="804">
@@ -18774,13 +19176,13 @@
         <v>1594</v>
       </c>
       <c r="B804" t="s">
-        <v>2298</v>
+        <v>2295</v>
       </c>
       <c r="C804" t="s">
-        <v>2299</v>
+        <v>2296</v>
       </c>
       <c r="D804" t="s">
-        <v>2300</v>
+        <v>2297</v>
       </c>
     </row>
     <row r="805">
@@ -18788,13 +19190,13 @@
         <v>1594</v>
       </c>
       <c r="B805" t="s">
-        <v>2301</v>
+        <v>2298</v>
       </c>
       <c r="C805" t="s">
-        <v>2302</v>
+        <v>2299</v>
       </c>
       <c r="D805" t="s">
-        <v>2303</v>
+        <v>2300</v>
       </c>
     </row>
     <row r="806">
@@ -18802,13 +19204,13 @@
         <v>1594</v>
       </c>
       <c r="B806" t="s">
-        <v>2304</v>
+        <v>2301</v>
       </c>
       <c r="C806" t="s">
-        <v>2305</v>
+        <v>2302</v>
       </c>
       <c r="D806" t="s">
-        <v>2306</v>
+        <v>2303</v>
       </c>
     </row>
     <row r="807">
@@ -18816,13 +19218,13 @@
         <v>1594</v>
       </c>
       <c r="B807" t="s">
-        <v>2307</v>
+        <v>2304</v>
       </c>
       <c r="C807" t="s">
-        <v>2308</v>
+        <v>2305</v>
       </c>
       <c r="D807" t="s">
-        <v>2309</v>
+        <v>2306</v>
       </c>
     </row>
     <row r="808">
@@ -18830,13 +19232,13 @@
         <v>1594</v>
       </c>
       <c r="B808" t="s">
-        <v>2310</v>
+        <v>2307</v>
       </c>
       <c r="C808" t="s">
-        <v>2311</v>
+        <v>2308</v>
       </c>
       <c r="D808" t="s">
-        <v>2312</v>
+        <v>2309</v>
       </c>
     </row>
     <row r="809">
@@ -18844,13 +19246,13 @@
         <v>1594</v>
       </c>
       <c r="B809" t="s">
-        <v>2313</v>
+        <v>2310</v>
       </c>
       <c r="C809" t="s">
-        <v>2109</v>
+        <v>2311</v>
       </c>
       <c r="D809" t="s">
-        <v>2110</v>
+        <v>2312</v>
       </c>
     </row>
     <row r="810">
@@ -18858,13 +19260,13 @@
         <v>1594</v>
       </c>
       <c r="B810" t="s">
+        <v>2313</v>
+      </c>
+      <c r="C810" t="s">
         <v>2314</v>
       </c>
-      <c r="C810" t="s">
+      <c r="D810" t="s">
         <v>2315</v>
-      </c>
-      <c r="D810" t="s">
-        <v>2316</v>
       </c>
     </row>
     <row r="811">
@@ -18872,13 +19274,13 @@
         <v>1594</v>
       </c>
       <c r="B811" t="s">
+        <v>2316</v>
+      </c>
+      <c r="C811" t="s">
         <v>2317</v>
       </c>
-      <c r="C811" t="s">
-        <v>2118</v>
-      </c>
       <c r="D811" t="s">
-        <v>2119</v>
+        <v>2318</v>
       </c>
     </row>
     <row r="812">
@@ -18886,13 +19288,13 @@
         <v>1594</v>
       </c>
       <c r="B812" t="s">
-        <v>2318</v>
+        <v>2319</v>
       </c>
       <c r="C812" t="s">
-        <v>2319</v>
+        <v>306</v>
       </c>
       <c r="D812" t="s">
-        <v>2320</v>
+        <v>307</v>
       </c>
     </row>
     <row r="813">
@@ -18900,13 +19302,13 @@
         <v>1594</v>
       </c>
       <c r="B813" t="s">
+        <v>2320</v>
+      </c>
+      <c r="C813" t="s">
         <v>2321</v>
       </c>
-      <c r="C813" t="s">
-        <v>2121</v>
-      </c>
       <c r="D813" t="s">
-        <v>2122</v>
+        <v>2322</v>
       </c>
     </row>
     <row r="814">
@@ -18914,13 +19316,13 @@
         <v>1594</v>
       </c>
       <c r="B814" t="s">
-        <v>2322</v>
+        <v>2323</v>
       </c>
       <c r="C814" t="s">
-        <v>2323</v>
+        <v>2324</v>
       </c>
       <c r="D814" t="s">
-        <v>2324</v>
+        <v>2325</v>
       </c>
     </row>
     <row r="815">
@@ -18928,13 +19330,13 @@
         <v>1594</v>
       </c>
       <c r="B815" t="s">
-        <v>2325</v>
+        <v>2326</v>
       </c>
       <c r="C815" t="s">
-        <v>2326</v>
+        <v>2327</v>
       </c>
       <c r="D815" t="s">
-        <v>2327</v>
+        <v>2328</v>
       </c>
     </row>
     <row r="816">
@@ -18942,13 +19344,13 @@
         <v>1594</v>
       </c>
       <c r="B816" t="s">
-        <v>2328</v>
+        <v>2329</v>
       </c>
       <c r="C816" t="s">
-        <v>2329</v>
+        <v>2330</v>
       </c>
       <c r="D816" t="s">
-        <v>2330</v>
+        <v>2331</v>
       </c>
     </row>
     <row r="817">
@@ -18956,13 +19358,13 @@
         <v>1594</v>
       </c>
       <c r="B817" t="s">
-        <v>2331</v>
+        <v>2332</v>
       </c>
       <c r="C817" t="s">
-        <v>2332</v>
+        <v>503</v>
       </c>
       <c r="D817" t="s">
-        <v>2333</v>
+        <v>504</v>
       </c>
     </row>
     <row r="818">
@@ -18970,13 +19372,13 @@
         <v>1594</v>
       </c>
       <c r="B818" t="s">
+        <v>2333</v>
+      </c>
+      <c r="C818" t="s">
         <v>2334</v>
       </c>
-      <c r="C818" t="s">
+      <c r="D818" t="s">
         <v>2335</v>
-      </c>
-      <c r="D818" t="s">
-        <v>2336</v>
       </c>
     </row>
     <row r="819">
@@ -18984,13 +19386,13 @@
         <v>1594</v>
       </c>
       <c r="B819" t="s">
+        <v>2336</v>
+      </c>
+      <c r="C819" t="s">
         <v>2337</v>
       </c>
-      <c r="C819" t="s">
+      <c r="D819" t="s">
         <v>2338</v>
-      </c>
-      <c r="D819" t="s">
-        <v>2339</v>
       </c>
     </row>
     <row r="820">
@@ -18998,13 +19400,13 @@
         <v>1594</v>
       </c>
       <c r="B820" t="s">
-        <v>2340</v>
+        <v>2339</v>
       </c>
       <c r="C820" t="s">
-        <v>1904</v>
+        <v>744</v>
       </c>
       <c r="D820" t="s">
-        <v>444</v>
+        <v>745</v>
       </c>
     </row>
     <row r="821">
@@ -19012,13 +19414,13 @@
         <v>1594</v>
       </c>
       <c r="B821" t="s">
+        <v>2340</v>
+      </c>
+      <c r="C821" t="s">
         <v>2341</v>
       </c>
-      <c r="C821" t="s">
+      <c r="D821" t="s">
         <v>2342</v>
-      </c>
-      <c r="D821" t="s">
-        <v>2343</v>
       </c>
     </row>
     <row r="822">
@@ -19026,13 +19428,13 @@
         <v>1594</v>
       </c>
       <c r="B822" t="s">
+        <v>2343</v>
+      </c>
+      <c r="C822" t="s">
         <v>2344</v>
       </c>
-      <c r="C822" t="s">
+      <c r="D822" t="s">
         <v>2345</v>
-      </c>
-      <c r="D822" t="s">
-        <v>2346</v>
       </c>
     </row>
     <row r="823">
@@ -19040,130 +19442,130 @@
         <v>1594</v>
       </c>
       <c r="B823" t="s">
+        <v>2346</v>
+      </c>
+      <c r="C823" t="s">
         <v>2347</v>
       </c>
-      <c r="C823" t="s">
+      <c r="D823" t="s">
         <v>2348</v>
-      </c>
-      <c r="D823" t="s">
-        <v>2349</v>
       </c>
     </row>
     <row r="824">
       <c r="A824" t="s">
-        <v>1609</v>
+        <v>1594</v>
       </c>
       <c r="B824" t="s">
+        <v>2349</v>
+      </c>
+      <c r="C824" t="s">
         <v>2350</v>
       </c>
-      <c r="C824" t="s">
-        <v>832</v>
-      </c>
       <c r="D824" t="s">
-        <v>833</v>
+        <v>2351</v>
       </c>
     </row>
     <row r="825">
       <c r="A825" t="s">
-        <v>1609</v>
+        <v>1594</v>
       </c>
       <c r="B825" t="s">
-        <v>2351</v>
+        <v>2352</v>
       </c>
       <c r="C825" t="s">
-        <v>2352</v>
+        <v>2353</v>
       </c>
       <c r="D825" t="s">
-        <v>2353</v>
+        <v>2354</v>
       </c>
     </row>
     <row r="826">
       <c r="A826" t="s">
-        <v>1609</v>
+        <v>1594</v>
       </c>
       <c r="B826" t="s">
-        <v>2354</v>
+        <v>2355</v>
       </c>
       <c r="C826" t="s">
-        <v>2355</v>
+        <v>2356</v>
       </c>
       <c r="D826" t="s">
-        <v>2356</v>
+        <v>2357</v>
       </c>
     </row>
     <row r="827">
       <c r="A827" t="s">
-        <v>2357</v>
+        <v>1594</v>
       </c>
       <c r="B827" t="s">
         <v>2358</v>
       </c>
       <c r="C827" t="s">
-        <v>2357</v>
+        <v>2359</v>
       </c>
       <c r="D827" t="s">
-        <v>2359</v>
+        <v>2360</v>
       </c>
     </row>
     <row r="828">
       <c r="A828" t="s">
-        <v>2357</v>
+        <v>1594</v>
       </c>
       <c r="B828" t="s">
-        <v>2360</v>
+        <v>2361</v>
       </c>
       <c r="C828" t="s">
-        <v>2361</v>
+        <v>2362</v>
       </c>
       <c r="D828" t="s">
-        <v>2362</v>
+        <v>2363</v>
       </c>
     </row>
     <row r="829">
       <c r="A829" t="s">
-        <v>2357</v>
+        <v>1594</v>
       </c>
       <c r="B829" t="s">
-        <v>2363</v>
+        <v>2364</v>
       </c>
       <c r="C829" t="s">
-        <v>2364</v>
+        <v>2365</v>
       </c>
       <c r="D829" t="s">
-        <v>2365</v>
+        <v>2366</v>
       </c>
     </row>
     <row r="830">
       <c r="A830" t="s">
-        <v>2357</v>
+        <v>1594</v>
       </c>
       <c r="B830" t="s">
-        <v>2366</v>
+        <v>2367</v>
       </c>
       <c r="C830" t="s">
-        <v>2367</v>
+        <v>2368</v>
       </c>
       <c r="D830" t="s">
-        <v>2368</v>
+        <v>2369</v>
       </c>
     </row>
     <row r="831">
       <c r="A831" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B831" t="s">
-        <v>2369</v>
+        <v>2370</v>
       </c>
       <c r="C831" t="s">
-        <v>2370</v>
+        <v>2371</v>
       </c>
       <c r="D831" t="s">
-        <v>2371</v>
+        <v>733</v>
       </c>
     </row>
     <row r="832">
       <c r="A832" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B832" t="s">
         <v>2372</v>
@@ -19177,7 +19579,7 @@
     </row>
     <row r="833">
       <c r="A833" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B833" t="s">
         <v>2375</v>
@@ -19191,133 +19593,133 @@
     </row>
     <row r="834">
       <c r="A834" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B834" t="s">
         <v>2378</v>
       </c>
       <c r="C834" t="s">
-        <v>280</v>
+        <v>2379</v>
       </c>
       <c r="D834" t="s">
-        <v>281</v>
+        <v>2380</v>
       </c>
     </row>
     <row r="835">
       <c r="A835" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B835" t="s">
-        <v>2379</v>
+        <v>2381</v>
       </c>
       <c r="C835" t="s">
-        <v>2380</v>
+        <v>2382</v>
       </c>
       <c r="D835" t="s">
-        <v>1764</v>
+        <v>2383</v>
       </c>
     </row>
     <row r="836">
       <c r="A836" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B836" t="s">
-        <v>2381</v>
+        <v>2384</v>
       </c>
       <c r="C836" t="s">
-        <v>2382</v>
+        <v>2385</v>
       </c>
       <c r="D836" t="s">
-        <v>2383</v>
+        <v>2386</v>
       </c>
     </row>
     <row r="837">
       <c r="A837" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B837" t="s">
-        <v>2384</v>
+        <v>2387</v>
       </c>
       <c r="C837" t="s">
-        <v>2385</v>
+        <v>2388</v>
       </c>
       <c r="D837" t="s">
-        <v>2386</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="838">
       <c r="A838" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B838" t="s">
-        <v>2387</v>
+        <v>2390</v>
       </c>
       <c r="C838" t="s">
-        <v>2388</v>
+        <v>2391</v>
       </c>
       <c r="D838" t="s">
-        <v>2389</v>
+        <v>2392</v>
       </c>
     </row>
     <row r="839">
       <c r="A839" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B839" t="s">
-        <v>2390</v>
+        <v>2393</v>
       </c>
       <c r="C839" t="s">
-        <v>2391</v>
+        <v>2394</v>
       </c>
       <c r="D839" t="s">
-        <v>2392</v>
+        <v>2395</v>
       </c>
     </row>
     <row r="840">
       <c r="A840" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B840" t="s">
-        <v>2393</v>
+        <v>2396</v>
       </c>
       <c r="C840" t="s">
-        <v>2394</v>
+        <v>2397</v>
       </c>
       <c r="D840" t="s">
-        <v>2395</v>
+        <v>142</v>
       </c>
     </row>
     <row r="841">
       <c r="A841" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B841" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="C841" t="s">
-        <v>2397</v>
+        <v>2399</v>
       </c>
       <c r="D841" t="s">
-        <v>2398</v>
+        <v>1557</v>
       </c>
     </row>
     <row r="842">
       <c r="A842" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B842" t="s">
-        <v>2399</v>
+        <v>2400</v>
       </c>
       <c r="C842" t="s">
-        <v>2400</v>
+        <v>2401</v>
       </c>
       <c r="D842" t="s">
-        <v>2401</v>
+        <v>1557</v>
       </c>
     </row>
     <row r="843">
       <c r="A843" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B843" t="s">
         <v>2402</v>
@@ -19331,7 +19733,7 @@
     </row>
     <row r="844">
       <c r="A844" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B844" t="s">
         <v>2405</v>
@@ -19345,7 +19747,7 @@
     </row>
     <row r="845">
       <c r="A845" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B845" t="s">
         <v>2408</v>
@@ -19359,7 +19761,7 @@
     </row>
     <row r="846">
       <c r="A846" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B846" t="s">
         <v>2411</v>
@@ -19373,7 +19775,7 @@
     </row>
     <row r="847">
       <c r="A847" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B847" t="s">
         <v>2414</v>
@@ -19387,189 +19789,189 @@
     </row>
     <row r="848">
       <c r="A848" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B848" t="s">
         <v>2417</v>
       </c>
       <c r="C848" t="s">
-        <v>2391</v>
+        <v>2418</v>
       </c>
       <c r="D848" t="s">
-        <v>2392</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="849">
       <c r="A849" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B849" t="s">
-        <v>2418</v>
+        <v>2420</v>
       </c>
       <c r="C849" t="s">
-        <v>2419</v>
+        <v>2421</v>
       </c>
       <c r="D849" t="s">
-        <v>2420</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="850">
       <c r="A850" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B850" t="s">
-        <v>2421</v>
+        <v>2423</v>
       </c>
       <c r="C850" t="s">
-        <v>2422</v>
+        <v>2424</v>
       </c>
       <c r="D850" t="s">
-        <v>2423</v>
+        <v>2425</v>
       </c>
     </row>
     <row r="851">
       <c r="A851" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B851" t="s">
-        <v>2424</v>
+        <v>2426</v>
       </c>
       <c r="C851" t="s">
-        <v>2425</v>
+        <v>2427</v>
       </c>
       <c r="D851" t="s">
-        <v>2426</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="852">
       <c r="A852" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B852" t="s">
-        <v>2427</v>
+        <v>2429</v>
       </c>
       <c r="C852" t="s">
-        <v>2428</v>
+        <v>2430</v>
       </c>
       <c r="D852" t="s">
-        <v>2429</v>
+        <v>2431</v>
       </c>
     </row>
     <row r="853">
       <c r="A853" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B853" t="s">
-        <v>2430</v>
+        <v>2432</v>
       </c>
       <c r="C853" t="s">
-        <v>2431</v>
+        <v>2433</v>
       </c>
       <c r="D853" t="s">
-        <v>2432</v>
+        <v>2434</v>
       </c>
     </row>
     <row r="854">
       <c r="A854" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B854" t="s">
-        <v>2433</v>
+        <v>2435</v>
       </c>
       <c r="C854" t="s">
-        <v>2434</v>
+        <v>2436</v>
       </c>
       <c r="D854" t="s">
-        <v>2435</v>
+        <v>2437</v>
       </c>
     </row>
     <row r="855">
       <c r="A855" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B855" t="s">
-        <v>2436</v>
+        <v>2438</v>
       </c>
       <c r="C855" t="s">
-        <v>2437</v>
+        <v>2439</v>
       </c>
       <c r="D855" t="s">
-        <v>2438</v>
+        <v>2440</v>
       </c>
     </row>
     <row r="856">
       <c r="A856" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B856" t="s">
-        <v>2439</v>
+        <v>2441</v>
       </c>
       <c r="C856" t="s">
-        <v>2440</v>
+        <v>2442</v>
       </c>
       <c r="D856" t="s">
-        <v>2441</v>
+        <v>2443</v>
       </c>
     </row>
     <row r="857">
       <c r="A857" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B857" t="s">
-        <v>2442</v>
+        <v>2444</v>
       </c>
       <c r="C857" t="s">
-        <v>2382</v>
+        <v>2445</v>
       </c>
       <c r="D857" t="s">
-        <v>2383</v>
+        <v>2446</v>
       </c>
     </row>
     <row r="858">
       <c r="A858" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B858" t="s">
-        <v>2443</v>
+        <v>2447</v>
       </c>
       <c r="C858" t="s">
-        <v>2444</v>
+        <v>2244</v>
       </c>
       <c r="D858" t="s">
-        <v>2445</v>
+        <v>2245</v>
       </c>
     </row>
     <row r="859">
       <c r="A859" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B859" t="s">
-        <v>2446</v>
+        <v>2448</v>
       </c>
       <c r="C859" t="s">
-        <v>2447</v>
+        <v>2449</v>
       </c>
       <c r="D859" t="s">
-        <v>2448</v>
+        <v>2450</v>
       </c>
     </row>
     <row r="860">
       <c r="A860" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B860" t="s">
-        <v>2449</v>
+        <v>2451</v>
       </c>
       <c r="C860" t="s">
-        <v>2450</v>
+        <v>2253</v>
       </c>
       <c r="D860" t="s">
-        <v>2451</v>
+        <v>2254</v>
       </c>
     </row>
     <row r="861">
       <c r="A861" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B861" t="s">
         <v>2452</v>
@@ -19583,91 +19985,91 @@
     </row>
     <row r="862">
       <c r="A862" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B862" t="s">
         <v>2455</v>
       </c>
       <c r="C862" t="s">
-        <v>2456</v>
+        <v>2256</v>
       </c>
       <c r="D862" t="s">
-        <v>2457</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="863">
       <c r="A863" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B863" t="s">
+        <v>2456</v>
+      </c>
+      <c r="C863" t="s">
+        <v>2457</v>
+      </c>
+      <c r="D863" t="s">
         <v>2458</v>
-      </c>
-      <c r="C863" t="s">
-        <v>2459</v>
-      </c>
-      <c r="D863" t="s">
-        <v>2460</v>
       </c>
     </row>
     <row r="864">
       <c r="A864" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B864" t="s">
+        <v>2459</v>
+      </c>
+      <c r="C864" t="s">
+        <v>2460</v>
+      </c>
+      <c r="D864" t="s">
         <v>2461</v>
-      </c>
-      <c r="C864" t="s">
-        <v>2462</v>
-      </c>
-      <c r="D864" t="s">
-        <v>2463</v>
       </c>
     </row>
     <row r="865">
       <c r="A865" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B865" t="s">
+        <v>2462</v>
+      </c>
+      <c r="C865" t="s">
+        <v>2463</v>
+      </c>
+      <c r="D865" t="s">
         <v>2464</v>
-      </c>
-      <c r="C865" t="s">
-        <v>2465</v>
-      </c>
-      <c r="D865" t="s">
-        <v>2466</v>
       </c>
     </row>
     <row r="866">
       <c r="A866" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B866" t="s">
+        <v>2465</v>
+      </c>
+      <c r="C866" t="s">
+        <v>2466</v>
+      </c>
+      <c r="D866" t="s">
         <v>2467</v>
-      </c>
-      <c r="C866" t="s">
-        <v>2468</v>
-      </c>
-      <c r="D866" t="s">
-        <v>2469</v>
       </c>
     </row>
     <row r="867">
       <c r="A867" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B867" t="s">
+        <v>2468</v>
+      </c>
+      <c r="C867" t="s">
+        <v>2469</v>
+      </c>
+      <c r="D867" t="s">
         <v>2470</v>
-      </c>
-      <c r="C867" t="s">
-        <v>1240</v>
-      </c>
-      <c r="D867" t="s">
-        <v>1241</v>
       </c>
     </row>
     <row r="868">
       <c r="A868" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B868" t="s">
         <v>2471</v>
@@ -19681,44 +20083,730 @@
     </row>
     <row r="869">
       <c r="A869" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B869" t="s">
         <v>2474</v>
       </c>
       <c r="C869" t="s">
-        <v>2475</v>
+        <v>1904</v>
       </c>
       <c r="D869" t="s">
-        <v>2476</v>
+        <v>444</v>
       </c>
     </row>
     <row r="870">
       <c r="A870" t="s">
-        <v>1612</v>
+        <v>1594</v>
       </c>
       <c r="B870" t="s">
+        <v>2475</v>
+      </c>
+      <c r="C870" t="s">
+        <v>2476</v>
+      </c>
+      <c r="D870" t="s">
         <v>2477</v>
-      </c>
-      <c r="C870" t="s">
-        <v>2478</v>
-      </c>
-      <c r="D870" t="s">
-        <v>2479</v>
       </c>
     </row>
     <row r="871">
       <c r="A871" t="s">
+        <v>1594</v>
+      </c>
+      <c r="B871" t="s">
+        <v>2478</v>
+      </c>
+      <c r="C871" t="s">
+        <v>2479</v>
+      </c>
+      <c r="D871" t="s">
+        <v>2480</v>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" t="s">
+        <v>1594</v>
+      </c>
+      <c r="B872" t="s">
+        <v>2481</v>
+      </c>
+      <c r="C872" t="s">
+        <v>2482</v>
+      </c>
+      <c r="D872" t="s">
+        <v>2483</v>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" t="s">
+        <v>1609</v>
+      </c>
+      <c r="B873" t="s">
+        <v>2484</v>
+      </c>
+      <c r="C873" t="s">
+        <v>832</v>
+      </c>
+      <c r="D873" t="s">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" t="s">
+        <v>1609</v>
+      </c>
+      <c r="B874" t="s">
+        <v>2485</v>
+      </c>
+      <c r="C874" t="s">
+        <v>2486</v>
+      </c>
+      <c r="D874" t="s">
+        <v>2487</v>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" t="s">
+        <v>1609</v>
+      </c>
+      <c r="B875" t="s">
+        <v>2488</v>
+      </c>
+      <c r="C875" t="s">
+        <v>2489</v>
+      </c>
+      <c r="D875" t="s">
+        <v>2490</v>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" t="s">
+        <v>2491</v>
+      </c>
+      <c r="B876" t="s">
+        <v>2492</v>
+      </c>
+      <c r="C876" t="s">
+        <v>2491</v>
+      </c>
+      <c r="D876" t="s">
+        <v>2493</v>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" t="s">
+        <v>2491</v>
+      </c>
+      <c r="B877" t="s">
+        <v>2494</v>
+      </c>
+      <c r="C877" t="s">
+        <v>2495</v>
+      </c>
+      <c r="D877" t="s">
+        <v>2496</v>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" t="s">
+        <v>2491</v>
+      </c>
+      <c r="B878" t="s">
+        <v>2497</v>
+      </c>
+      <c r="C878" t="s">
+        <v>2498</v>
+      </c>
+      <c r="D878" t="s">
+        <v>2499</v>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" t="s">
+        <v>2491</v>
+      </c>
+      <c r="B879" t="s">
+        <v>2500</v>
+      </c>
+      <c r="C879" t="s">
+        <v>2501</v>
+      </c>
+      <c r="D879" t="s">
+        <v>2502</v>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" t="s">
         <v>1612</v>
       </c>
-      <c r="B871" t="s">
-        <v>2480</v>
-      </c>
-      <c r="C871" t="s">
-        <v>2481</v>
-      </c>
-      <c r="D871" t="s">
-        <v>2482</v>
+      <c r="B880" t="s">
+        <v>2503</v>
+      </c>
+      <c r="C880" t="s">
+        <v>2504</v>
+      </c>
+      <c r="D880" t="s">
+        <v>2505</v>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B881" t="s">
+        <v>2506</v>
+      </c>
+      <c r="C881" t="s">
+        <v>2507</v>
+      </c>
+      <c r="D881" t="s">
+        <v>2508</v>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B882" t="s">
+        <v>2509</v>
+      </c>
+      <c r="C882" t="s">
+        <v>2510</v>
+      </c>
+      <c r="D882" t="s">
+        <v>2511</v>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B883" t="s">
+        <v>2512</v>
+      </c>
+      <c r="C883" t="s">
+        <v>280</v>
+      </c>
+      <c r="D883" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B884" t="s">
+        <v>2513</v>
+      </c>
+      <c r="C884" t="s">
+        <v>2514</v>
+      </c>
+      <c r="D884" t="s">
+        <v>1764</v>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B885" t="s">
+        <v>2515</v>
+      </c>
+      <c r="C885" t="s">
+        <v>2516</v>
+      </c>
+      <c r="D885" t="s">
+        <v>2517</v>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B886" t="s">
+        <v>2518</v>
+      </c>
+      <c r="C886" t="s">
+        <v>2519</v>
+      </c>
+      <c r="D886" t="s">
+        <v>2520</v>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B887" t="s">
+        <v>2521</v>
+      </c>
+      <c r="C887" t="s">
+        <v>2522</v>
+      </c>
+      <c r="D887" t="s">
+        <v>2523</v>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B888" t="s">
+        <v>2524</v>
+      </c>
+      <c r="C888" t="s">
+        <v>2525</v>
+      </c>
+      <c r="D888" t="s">
+        <v>2526</v>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B889" t="s">
+        <v>2527</v>
+      </c>
+      <c r="C889" t="s">
+        <v>2528</v>
+      </c>
+      <c r="D889" t="s">
+        <v>2529</v>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B890" t="s">
+        <v>2530</v>
+      </c>
+      <c r="C890" t="s">
+        <v>2531</v>
+      </c>
+      <c r="D890" t="s">
+        <v>2532</v>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B891" t="s">
+        <v>2533</v>
+      </c>
+      <c r="C891" t="s">
+        <v>2534</v>
+      </c>
+      <c r="D891" t="s">
+        <v>2535</v>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B892" t="s">
+        <v>2536</v>
+      </c>
+      <c r="C892" t="s">
+        <v>2537</v>
+      </c>
+      <c r="D892" t="s">
+        <v>2538</v>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B893" t="s">
+        <v>2539</v>
+      </c>
+      <c r="C893" t="s">
+        <v>2540</v>
+      </c>
+      <c r="D893" t="s">
+        <v>2541</v>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B894" t="s">
+        <v>2542</v>
+      </c>
+      <c r="C894" t="s">
+        <v>2543</v>
+      </c>
+      <c r="D894" t="s">
+        <v>2544</v>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B895" t="s">
+        <v>2545</v>
+      </c>
+      <c r="C895" t="s">
+        <v>2546</v>
+      </c>
+      <c r="D895" t="s">
+        <v>2547</v>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B896" t="s">
+        <v>2548</v>
+      </c>
+      <c r="C896" t="s">
+        <v>2549</v>
+      </c>
+      <c r="D896" t="s">
+        <v>2550</v>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B897" t="s">
+        <v>2551</v>
+      </c>
+      <c r="C897" t="s">
+        <v>2525</v>
+      </c>
+      <c r="D897" t="s">
+        <v>2526</v>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B898" t="s">
+        <v>2552</v>
+      </c>
+      <c r="C898" t="s">
+        <v>2553</v>
+      </c>
+      <c r="D898" t="s">
+        <v>2554</v>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B899" t="s">
+        <v>2555</v>
+      </c>
+      <c r="C899" t="s">
+        <v>2556</v>
+      </c>
+      <c r="D899" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B900" t="s">
+        <v>2558</v>
+      </c>
+      <c r="C900" t="s">
+        <v>2559</v>
+      </c>
+      <c r="D900" t="s">
+        <v>2560</v>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B901" t="s">
+        <v>2561</v>
+      </c>
+      <c r="C901" t="s">
+        <v>2562</v>
+      </c>
+      <c r="D901" t="s">
+        <v>2563</v>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B902" t="s">
+        <v>2564</v>
+      </c>
+      <c r="C902" t="s">
+        <v>2565</v>
+      </c>
+      <c r="D902" t="s">
+        <v>2566</v>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B903" t="s">
+        <v>2567</v>
+      </c>
+      <c r="C903" t="s">
+        <v>2568</v>
+      </c>
+      <c r="D903" t="s">
+        <v>2569</v>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B904" t="s">
+        <v>2570</v>
+      </c>
+      <c r="C904" t="s">
+        <v>2571</v>
+      </c>
+      <c r="D904" t="s">
+        <v>2572</v>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B905" t="s">
+        <v>2573</v>
+      </c>
+      <c r="C905" t="s">
+        <v>2574</v>
+      </c>
+      <c r="D905" t="s">
+        <v>2575</v>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B906" t="s">
+        <v>2576</v>
+      </c>
+      <c r="C906" t="s">
+        <v>2516</v>
+      </c>
+      <c r="D906" t="s">
+        <v>2517</v>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B907" t="s">
+        <v>2577</v>
+      </c>
+      <c r="C907" t="s">
+        <v>2578</v>
+      </c>
+      <c r="D907" t="s">
+        <v>2579</v>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B908" t="s">
+        <v>2580</v>
+      </c>
+      <c r="C908" t="s">
+        <v>2581</v>
+      </c>
+      <c r="D908" t="s">
+        <v>2582</v>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B909" t="s">
+        <v>2583</v>
+      </c>
+      <c r="C909" t="s">
+        <v>2584</v>
+      </c>
+      <c r="D909" t="s">
+        <v>2585</v>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B910" t="s">
+        <v>2586</v>
+      </c>
+      <c r="C910" t="s">
+        <v>2587</v>
+      </c>
+      <c r="D910" t="s">
+        <v>2588</v>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B911" t="s">
+        <v>2589</v>
+      </c>
+      <c r="C911" t="s">
+        <v>2590</v>
+      </c>
+      <c r="D911" t="s">
+        <v>2591</v>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B912" t="s">
+        <v>2592</v>
+      </c>
+      <c r="C912" t="s">
+        <v>2593</v>
+      </c>
+      <c r="D912" t="s">
+        <v>2594</v>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B913" t="s">
+        <v>2595</v>
+      </c>
+      <c r="C913" t="s">
+        <v>2596</v>
+      </c>
+      <c r="D913" t="s">
+        <v>2597</v>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B914" t="s">
+        <v>2598</v>
+      </c>
+      <c r="C914" t="s">
+        <v>2599</v>
+      </c>
+      <c r="D914" t="s">
+        <v>2600</v>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B915" t="s">
+        <v>2601</v>
+      </c>
+      <c r="C915" t="s">
+        <v>2602</v>
+      </c>
+      <c r="D915" t="s">
+        <v>2603</v>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B916" t="s">
+        <v>2604</v>
+      </c>
+      <c r="C916" t="s">
+        <v>1240</v>
+      </c>
+      <c r="D916" t="s">
+        <v>1241</v>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B917" t="s">
+        <v>2605</v>
+      </c>
+      <c r="C917" t="s">
+        <v>2606</v>
+      </c>
+      <c r="D917" t="s">
+        <v>2607</v>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B918" t="s">
+        <v>2608</v>
+      </c>
+      <c r="C918" t="s">
+        <v>2609</v>
+      </c>
+      <c r="D918" t="s">
+        <v>2610</v>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B919" t="s">
+        <v>2611</v>
+      </c>
+      <c r="C919" t="s">
+        <v>2612</v>
+      </c>
+      <c r="D919" t="s">
+        <v>2613</v>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B920" t="s">
+        <v>2614</v>
+      </c>
+      <c r="C920" t="s">
+        <v>2615</v>
+      </c>
+      <c r="D920" t="s">
+        <v>2616</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Accessibility: heading order on import, labels on revenue month fields
</commit_message>
<xml_diff>
--- a/docs/amharic-review.xlsx
+++ b/docs/amharic-review.xlsx
@@ -6364,6 +6364,15 @@
     <t>የውል ማብቂያ</t>
   </si>
   <si>
+    <t>rep.fromMonth</t>
+  </si>
+  <si>
+    <t>From month</t>
+  </si>
+  <si>
+    <t>ከወር</t>
+  </si>
+  <si>
     <t>rep.k.bestMonth</t>
   </si>
   <si>
@@ -6749,6 +6758,15 @@
   </si>
   <si>
     <t>የቀረ ጊዜ</t>
+  </si>
+  <si>
+    <t>rep.toMonth</t>
+  </si>
+  <si>
+    <t>To month</t>
+  </si>
+  <si>
+    <t>እስከ ወር</t>
   </si>
   <si>
     <t>rep.toReturn</t>
@@ -18675,10 +18693,10 @@
         <v>2119</v>
       </c>
       <c r="C741" t="s">
-        <v>21</v>
+        <v>2120</v>
       </c>
       <c r="D741" t="s">
-        <v>2120</v>
+        <v>2121</v>
       </c>
     </row>
     <row r="742">
@@ -18686,10 +18704,10 @@
         <v>1724</v>
       </c>
       <c r="B742" t="s">
-        <v>2121</v>
+        <v>2122</v>
       </c>
       <c r="C742" t="s">
-        <v>2122</v>
+        <v>21</v>
       </c>
       <c r="D742" t="s">
         <v>2123</v>
@@ -18734,7 +18752,7 @@
         <v>2131</v>
       </c>
       <c r="D745" t="s">
-        <v>2090</v>
+        <v>2132</v>
       </c>
     </row>
     <row r="746">
@@ -18742,13 +18760,13 @@
         <v>1724</v>
       </c>
       <c r="B746" t="s">
-        <v>2132</v>
+        <v>2133</v>
       </c>
       <c r="C746" t="s">
-        <v>2133</v>
+        <v>2134</v>
       </c>
       <c r="D746" t="s">
-        <v>2134</v>
+        <v>2090</v>
       </c>
     </row>
     <row r="747">
@@ -18815,10 +18833,10 @@
         <v>2147</v>
       </c>
       <c r="C751" t="s">
-        <v>1208</v>
+        <v>2148</v>
       </c>
       <c r="D751" t="s">
-        <v>2148</v>
+        <v>2149</v>
       </c>
     </row>
     <row r="752">
@@ -18826,10 +18844,10 @@
         <v>1724</v>
       </c>
       <c r="B752" t="s">
-        <v>2149</v>
+        <v>2150</v>
       </c>
       <c r="C752" t="s">
-        <v>2150</v>
+        <v>1208</v>
       </c>
       <c r="D752" t="s">
         <v>2151</v>
@@ -18843,10 +18861,10 @@
         <v>2152</v>
       </c>
       <c r="C753" t="s">
-        <v>381</v>
+        <v>2153</v>
       </c>
       <c r="D753" t="s">
-        <v>2153</v>
+        <v>2154</v>
       </c>
     </row>
     <row r="754">
@@ -18854,10 +18872,10 @@
         <v>1724</v>
       </c>
       <c r="B754" t="s">
-        <v>2154</v>
+        <v>2155</v>
       </c>
       <c r="C754" t="s">
-        <v>2155</v>
+        <v>381</v>
       </c>
       <c r="D754" t="s">
         <v>2156</v>
@@ -18941,10 +18959,10 @@
         <v>2172</v>
       </c>
       <c r="C760" t="s">
-        <v>376</v>
+        <v>2173</v>
       </c>
       <c r="D760" t="s">
-        <v>2173</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="761">
@@ -18952,13 +18970,13 @@
         <v>1724</v>
       </c>
       <c r="B761" t="s">
-        <v>2174</v>
+        <v>2175</v>
       </c>
       <c r="C761" t="s">
-        <v>393</v>
+        <v>376</v>
       </c>
       <c r="D761" t="s">
-        <v>394</v>
+        <v>2176</v>
       </c>
     </row>
     <row r="762">
@@ -18966,13 +18984,13 @@
         <v>1724</v>
       </c>
       <c r="B762" t="s">
-        <v>2175</v>
+        <v>2177</v>
       </c>
       <c r="C762" t="s">
-        <v>2176</v>
+        <v>393</v>
       </c>
       <c r="D762" t="s">
-        <v>2173</v>
+        <v>394</v>
       </c>
     </row>
     <row r="763">
@@ -18980,13 +18998,13 @@
         <v>1724</v>
       </c>
       <c r="B763" t="s">
-        <v>2177</v>
+        <v>2178</v>
       </c>
       <c r="C763" t="s">
-        <v>2178</v>
+        <v>2179</v>
       </c>
       <c r="D763" t="s">
-        <v>2179</v>
+        <v>2176</v>
       </c>
     </row>
     <row r="764">
@@ -19070,7 +19088,7 @@
         <v>2196</v>
       </c>
       <c r="D769" t="s">
-        <v>2126</v>
+        <v>2197</v>
       </c>
     </row>
     <row r="770">
@@ -19078,13 +19096,13 @@
         <v>1724</v>
       </c>
       <c r="B770" t="s">
-        <v>2197</v>
+        <v>2198</v>
       </c>
       <c r="C770" t="s">
-        <v>2198</v>
+        <v>2199</v>
       </c>
       <c r="D770" t="s">
-        <v>2199</v>
+        <v>2129</v>
       </c>
     </row>
     <row r="771">
@@ -19098,7 +19116,7 @@
         <v>2201</v>
       </c>
       <c r="D771" t="s">
-        <v>1666</v>
+        <v>2202</v>
       </c>
     </row>
     <row r="772">
@@ -19106,13 +19124,13 @@
         <v>1724</v>
       </c>
       <c r="B772" t="s">
-        <v>2202</v>
+        <v>2203</v>
       </c>
       <c r="C772" t="s">
-        <v>2203</v>
+        <v>2204</v>
       </c>
       <c r="D772" t="s">
-        <v>2204</v>
+        <v>1666</v>
       </c>
     </row>
     <row r="773">
@@ -19154,7 +19172,7 @@
         <v>2212</v>
       </c>
       <c r="D775" t="s">
-        <v>1412</v>
+        <v>2213</v>
       </c>
     </row>
     <row r="776">
@@ -19162,13 +19180,13 @@
         <v>1724</v>
       </c>
       <c r="B776" t="s">
-        <v>2213</v>
+        <v>2214</v>
       </c>
       <c r="C776" t="s">
-        <v>2214</v>
+        <v>2215</v>
       </c>
       <c r="D776" t="s">
-        <v>2215</v>
+        <v>1412</v>
       </c>
     </row>
     <row r="777">
@@ -19179,10 +19197,10 @@
         <v>2216</v>
       </c>
       <c r="C777" t="s">
-        <v>1735</v>
+        <v>2217</v>
       </c>
       <c r="D777" t="s">
-        <v>1750</v>
+        <v>2218</v>
       </c>
     </row>
     <row r="778">
@@ -19190,13 +19208,13 @@
         <v>1724</v>
       </c>
       <c r="B778" t="s">
-        <v>2217</v>
+        <v>2219</v>
       </c>
       <c r="C778" t="s">
-        <v>48</v>
+        <v>1735</v>
       </c>
       <c r="D778" t="s">
-        <v>49</v>
+        <v>1750</v>
       </c>
     </row>
     <row r="779">
@@ -19204,13 +19222,13 @@
         <v>1724</v>
       </c>
       <c r="B779" t="s">
-        <v>2218</v>
+        <v>2220</v>
       </c>
       <c r="C779" t="s">
-        <v>2219</v>
+        <v>48</v>
       </c>
       <c r="D779" t="s">
-        <v>2220</v>
+        <v>49</v>
       </c>
     </row>
     <row r="780">
@@ -19383,35 +19401,35 @@
     </row>
     <row r="792">
       <c r="A792" t="s">
+        <v>1724</v>
+      </c>
+      <c r="B792" t="s">
         <v>2257</v>
       </c>
-      <c r="B792" t="s">
+      <c r="C792" t="s">
         <v>2258</v>
       </c>
-      <c r="C792" t="s">
+      <c r="D792" t="s">
         <v>2259</v>
-      </c>
-      <c r="D792" t="s">
-        <v>2260</v>
       </c>
     </row>
     <row r="793">
       <c r="A793" t="s">
-        <v>2257</v>
+        <v>1724</v>
       </c>
       <c r="B793" t="s">
+        <v>2260</v>
+      </c>
+      <c r="C793" t="s">
         <v>2261</v>
       </c>
-      <c r="C793" t="s">
+      <c r="D793" t="s">
         <v>2262</v>
-      </c>
-      <c r="D793" t="s">
-        <v>2263</v>
       </c>
     </row>
     <row r="794">
       <c r="A794" t="s">
-        <v>2257</v>
+        <v>2263</v>
       </c>
       <c r="B794" t="s">
         <v>2264</v>
@@ -19425,7 +19443,7 @@
     </row>
     <row r="795">
       <c r="A795" t="s">
-        <v>2257</v>
+        <v>2263</v>
       </c>
       <c r="B795" t="s">
         <v>2267</v>
@@ -19439,7 +19457,7 @@
     </row>
     <row r="796">
       <c r="A796" t="s">
-        <v>1338</v>
+        <v>2263</v>
       </c>
       <c r="B796" t="s">
         <v>2270</v>
@@ -19453,7 +19471,7 @@
     </row>
     <row r="797">
       <c r="A797" t="s">
-        <v>1338</v>
+        <v>2263</v>
       </c>
       <c r="B797" t="s">
         <v>2273</v>
@@ -19481,7 +19499,7 @@
     </row>
     <row r="799">
       <c r="A799" t="s">
-        <v>1715</v>
+        <v>1338</v>
       </c>
       <c r="B799" t="s">
         <v>2279</v>
@@ -19495,7 +19513,7 @@
     </row>
     <row r="800">
       <c r="A800" t="s">
-        <v>1715</v>
+        <v>1338</v>
       </c>
       <c r="B800" t="s">
         <v>2282</v>
@@ -20005,10 +20023,10 @@
         <v>2390</v>
       </c>
       <c r="C836" t="s">
-        <v>967</v>
+        <v>2391</v>
       </c>
       <c r="D836" t="s">
-        <v>2182</v>
+        <v>2392</v>
       </c>
     </row>
     <row r="837">
@@ -20016,13 +20034,13 @@
         <v>1715</v>
       </c>
       <c r="B837" t="s">
-        <v>2391</v>
+        <v>2393</v>
       </c>
       <c r="C837" t="s">
-        <v>2392</v>
+        <v>2394</v>
       </c>
       <c r="D837" t="s">
-        <v>2393</v>
+        <v>2395</v>
       </c>
     </row>
     <row r="838">
@@ -20030,13 +20048,13 @@
         <v>1715</v>
       </c>
       <c r="B838" t="s">
-        <v>2394</v>
+        <v>2396</v>
       </c>
       <c r="C838" t="s">
-        <v>2395</v>
+        <v>967</v>
       </c>
       <c r="D838" t="s">
-        <v>2396</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="839">
@@ -20271,10 +20289,10 @@
         <v>2445</v>
       </c>
       <c r="C855" t="s">
-        <v>330</v>
+        <v>2446</v>
       </c>
       <c r="D855" t="s">
-        <v>331</v>
+        <v>2447</v>
       </c>
     </row>
     <row r="856">
@@ -20282,13 +20300,13 @@
         <v>1715</v>
       </c>
       <c r="B856" t="s">
-        <v>2446</v>
+        <v>2448</v>
       </c>
       <c r="C856" t="s">
-        <v>2447</v>
+        <v>2449</v>
       </c>
       <c r="D856" t="s">
-        <v>2448</v>
+        <v>2450</v>
       </c>
     </row>
     <row r="857">
@@ -20296,13 +20314,13 @@
         <v>1715</v>
       </c>
       <c r="B857" t="s">
-        <v>2449</v>
+        <v>2451</v>
       </c>
       <c r="C857" t="s">
-        <v>2450</v>
+        <v>330</v>
       </c>
       <c r="D857" t="s">
-        <v>2451</v>
+        <v>331</v>
       </c>
     </row>
     <row r="858">
@@ -20341,10 +20359,10 @@
         <v>2458</v>
       </c>
       <c r="C860" t="s">
-        <v>545</v>
+        <v>2459</v>
       </c>
       <c r="D860" t="s">
-        <v>546</v>
+        <v>2460</v>
       </c>
     </row>
     <row r="861">
@@ -20352,13 +20370,13 @@
         <v>1715</v>
       </c>
       <c r="B861" t="s">
-        <v>2459</v>
+        <v>2461</v>
       </c>
       <c r="C861" t="s">
-        <v>2460</v>
+        <v>2462</v>
       </c>
       <c r="D861" t="s">
-        <v>2461</v>
+        <v>2463</v>
       </c>
     </row>
     <row r="862">
@@ -20366,13 +20384,13 @@
         <v>1715</v>
       </c>
       <c r="B862" t="s">
-        <v>2462</v>
+        <v>2464</v>
       </c>
       <c r="C862" t="s">
-        <v>2463</v>
+        <v>545</v>
       </c>
       <c r="D862" t="s">
-        <v>2464</v>
+        <v>546</v>
       </c>
     </row>
     <row r="863">
@@ -20383,10 +20401,10 @@
         <v>2465</v>
       </c>
       <c r="C863" t="s">
-        <v>786</v>
+        <v>2466</v>
       </c>
       <c r="D863" t="s">
-        <v>787</v>
+        <v>2467</v>
       </c>
     </row>
     <row r="864">
@@ -20394,13 +20412,13 @@
         <v>1715</v>
       </c>
       <c r="B864" t="s">
-        <v>2466</v>
+        <v>2468</v>
       </c>
       <c r="C864" t="s">
-        <v>2467</v>
+        <v>2469</v>
       </c>
       <c r="D864" t="s">
-        <v>2468</v>
+        <v>2470</v>
       </c>
     </row>
     <row r="865">
@@ -20408,13 +20426,13 @@
         <v>1715</v>
       </c>
       <c r="B865" t="s">
-        <v>2469</v>
+        <v>2471</v>
       </c>
       <c r="C865" t="s">
-        <v>2470</v>
+        <v>786</v>
       </c>
       <c r="D865" t="s">
-        <v>2471</v>
+        <v>787</v>
       </c>
     </row>
     <row r="866">
@@ -20540,7 +20558,7 @@
         <v>2497</v>
       </c>
       <c r="D874" t="s">
-        <v>775</v>
+        <v>2498</v>
       </c>
     </row>
     <row r="875">
@@ -20548,13 +20566,13 @@
         <v>1715</v>
       </c>
       <c r="B875" t="s">
-        <v>2498</v>
+        <v>2499</v>
       </c>
       <c r="C875" t="s">
-        <v>2499</v>
+        <v>2500</v>
       </c>
       <c r="D875" t="s">
-        <v>2500</v>
+        <v>2501</v>
       </c>
     </row>
     <row r="876">
@@ -20562,13 +20580,13 @@
         <v>1715</v>
       </c>
       <c r="B876" t="s">
-        <v>2501</v>
+        <v>2502</v>
       </c>
       <c r="C876" t="s">
-        <v>2502</v>
+        <v>2503</v>
       </c>
       <c r="D876" t="s">
-        <v>2503</v>
+        <v>775</v>
       </c>
     </row>
     <row r="877">
@@ -20666,7 +20684,7 @@
         <v>2523</v>
       </c>
       <c r="D883" t="s">
-        <v>166</v>
+        <v>2524</v>
       </c>
     </row>
     <row r="884">
@@ -20674,13 +20692,13 @@
         <v>1715</v>
       </c>
       <c r="B884" t="s">
-        <v>2524</v>
+        <v>2525</v>
       </c>
       <c r="C884" t="s">
-        <v>2525</v>
+        <v>2526</v>
       </c>
       <c r="D884" t="s">
-        <v>1666</v>
+        <v>2527</v>
       </c>
     </row>
     <row r="885">
@@ -20688,13 +20706,13 @@
         <v>1715</v>
       </c>
       <c r="B885" t="s">
-        <v>2526</v>
+        <v>2528</v>
       </c>
       <c r="C885" t="s">
-        <v>2527</v>
+        <v>2529</v>
       </c>
       <c r="D885" t="s">
-        <v>1666</v>
+        <v>166</v>
       </c>
     </row>
     <row r="886">
@@ -20702,13 +20720,13 @@
         <v>1715</v>
       </c>
       <c r="B886" t="s">
-        <v>2528</v>
+        <v>2530</v>
       </c>
       <c r="C886" t="s">
-        <v>2529</v>
+        <v>2531</v>
       </c>
       <c r="D886" t="s">
-        <v>2530</v>
+        <v>1666</v>
       </c>
     </row>
     <row r="887">
@@ -20716,13 +20734,13 @@
         <v>1715</v>
       </c>
       <c r="B887" t="s">
-        <v>2531</v>
+        <v>2532</v>
       </c>
       <c r="C887" t="s">
-        <v>2532</v>
+        <v>2533</v>
       </c>
       <c r="D887" t="s">
-        <v>2533</v>
+        <v>1666</v>
       </c>
     </row>
     <row r="888">
@@ -20915,10 +20933,10 @@
         <v>2573</v>
       </c>
       <c r="C901" t="s">
-        <v>2370</v>
+        <v>2574</v>
       </c>
       <c r="D901" t="s">
-        <v>2371</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="902">
@@ -20926,13 +20944,13 @@
         <v>1715</v>
       </c>
       <c r="B902" t="s">
-        <v>2574</v>
+        <v>2576</v>
       </c>
       <c r="C902" t="s">
-        <v>2575</v>
+        <v>2577</v>
       </c>
       <c r="D902" t="s">
-        <v>2576</v>
+        <v>2578</v>
       </c>
     </row>
     <row r="903">
@@ -20940,13 +20958,13 @@
         <v>1715</v>
       </c>
       <c r="B903" t="s">
-        <v>2577</v>
+        <v>2579</v>
       </c>
       <c r="C903" t="s">
-        <v>2379</v>
+        <v>2376</v>
       </c>
       <c r="D903" t="s">
-        <v>2380</v>
+        <v>2377</v>
       </c>
     </row>
     <row r="904">
@@ -20954,13 +20972,13 @@
         <v>1715</v>
       </c>
       <c r="B904" t="s">
-        <v>2578</v>
+        <v>2580</v>
       </c>
       <c r="C904" t="s">
-        <v>2579</v>
+        <v>2581</v>
       </c>
       <c r="D904" t="s">
-        <v>2580</v>
+        <v>2582</v>
       </c>
     </row>
     <row r="905">
@@ -20968,13 +20986,13 @@
         <v>1715</v>
       </c>
       <c r="B905" t="s">
-        <v>2581</v>
+        <v>2583</v>
       </c>
       <c r="C905" t="s">
-        <v>2382</v>
+        <v>2385</v>
       </c>
       <c r="D905" t="s">
-        <v>2383</v>
+        <v>2386</v>
       </c>
     </row>
     <row r="906">
@@ -20982,13 +21000,13 @@
         <v>1715</v>
       </c>
       <c r="B906" t="s">
-        <v>2582</v>
+        <v>2584</v>
       </c>
       <c r="C906" t="s">
-        <v>2583</v>
+        <v>2585</v>
       </c>
       <c r="D906" t="s">
-        <v>2584</v>
+        <v>2586</v>
       </c>
     </row>
     <row r="907">
@@ -20996,13 +21014,13 @@
         <v>1715</v>
       </c>
       <c r="B907" t="s">
-        <v>2585</v>
+        <v>2587</v>
       </c>
       <c r="C907" t="s">
-        <v>2586</v>
+        <v>2388</v>
       </c>
       <c r="D907" t="s">
-        <v>2587</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="908">
@@ -21069,10 +21087,10 @@
         <v>2600</v>
       </c>
       <c r="C912" t="s">
-        <v>2025</v>
+        <v>2601</v>
       </c>
       <c r="D912" t="s">
-        <v>474</v>
+        <v>2602</v>
       </c>
     </row>
     <row r="913">
@@ -21080,13 +21098,13 @@
         <v>1715</v>
       </c>
       <c r="B913" t="s">
-        <v>2601</v>
+        <v>2603</v>
       </c>
       <c r="C913" t="s">
-        <v>2602</v>
+        <v>2604</v>
       </c>
       <c r="D913" t="s">
-        <v>2603</v>
+        <v>2605</v>
       </c>
     </row>
     <row r="914">
@@ -21094,13 +21112,13 @@
         <v>1715</v>
       </c>
       <c r="B914" t="s">
-        <v>2604</v>
+        <v>2606</v>
       </c>
       <c r="C914" t="s">
-        <v>2605</v>
+        <v>2025</v>
       </c>
       <c r="D914" t="s">
-        <v>2606</v>
+        <v>474</v>
       </c>
     </row>
     <row r="915">
@@ -21119,30 +21137,30 @@
     </row>
     <row r="916">
       <c r="A916" t="s">
-        <v>1730</v>
+        <v>1715</v>
       </c>
       <c r="B916" t="s">
         <v>2610</v>
       </c>
       <c r="C916" t="s">
-        <v>874</v>
+        <v>2611</v>
       </c>
       <c r="D916" t="s">
-        <v>875</v>
+        <v>2612</v>
       </c>
     </row>
     <row r="917">
       <c r="A917" t="s">
-        <v>1730</v>
+        <v>1715</v>
       </c>
       <c r="B917" t="s">
-        <v>2611</v>
+        <v>2613</v>
       </c>
       <c r="C917" t="s">
-        <v>2612</v>
+        <v>2614</v>
       </c>
       <c r="D917" t="s">
-        <v>2613</v>
+        <v>2615</v>
       </c>
     </row>
     <row r="918">
@@ -21150,24 +21168,24 @@
         <v>1730</v>
       </c>
       <c r="B918" t="s">
-        <v>2614</v>
+        <v>2616</v>
       </c>
       <c r="C918" t="s">
-        <v>2615</v>
+        <v>874</v>
       </c>
       <c r="D918" t="s">
-        <v>2616</v>
+        <v>875</v>
       </c>
     </row>
     <row r="919">
       <c r="A919" t="s">
+        <v>1730</v>
+      </c>
+      <c r="B919" t="s">
         <v>2617</v>
       </c>
-      <c r="B919" t="s">
+      <c r="C919" t="s">
         <v>2618</v>
-      </c>
-      <c r="C919" t="s">
-        <v>2617</v>
       </c>
       <c r="D919" t="s">
         <v>2619</v>
@@ -21175,7 +21193,7 @@
     </row>
     <row r="920">
       <c r="A920" t="s">
-        <v>2617</v>
+        <v>1730</v>
       </c>
       <c r="B920" t="s">
         <v>2620</v>
@@ -21189,13 +21207,13 @@
     </row>
     <row r="921">
       <c r="A921" t="s">
-        <v>2617</v>
+        <v>2623</v>
       </c>
       <c r="B921" t="s">
+        <v>2624</v>
+      </c>
+      <c r="C921" t="s">
         <v>2623</v>
-      </c>
-      <c r="C921" t="s">
-        <v>2624</v>
       </c>
       <c r="D921" t="s">
         <v>2625</v>
@@ -21203,7 +21221,7 @@
     </row>
     <row r="922">
       <c r="A922" t="s">
-        <v>2617</v>
+        <v>2623</v>
       </c>
       <c r="B922" t="s">
         <v>2626</v>
@@ -21217,7 +21235,7 @@
     </row>
     <row r="923">
       <c r="A923" t="s">
-        <v>1733</v>
+        <v>2623</v>
       </c>
       <c r="B923" t="s">
         <v>2629</v>
@@ -21231,7 +21249,7 @@
     </row>
     <row r="924">
       <c r="A924" t="s">
-        <v>1733</v>
+        <v>2623</v>
       </c>
       <c r="B924" t="s">
         <v>2632</v>
@@ -21265,10 +21283,10 @@
         <v>2638</v>
       </c>
       <c r="C926" t="s">
-        <v>304</v>
+        <v>2639</v>
       </c>
       <c r="D926" t="s">
-        <v>305</v>
+        <v>2640</v>
       </c>
     </row>
     <row r="927">
@@ -21276,13 +21294,13 @@
         <v>1733</v>
       </c>
       <c r="B927" t="s">
-        <v>2639</v>
+        <v>2641</v>
       </c>
       <c r="C927" t="s">
-        <v>2640</v>
+        <v>2642</v>
       </c>
       <c r="D927" t="s">
-        <v>1885</v>
+        <v>2643</v>
       </c>
     </row>
     <row r="928">
@@ -21290,13 +21308,13 @@
         <v>1733</v>
       </c>
       <c r="B928" t="s">
-        <v>2641</v>
+        <v>2644</v>
       </c>
       <c r="C928" t="s">
-        <v>2642</v>
+        <v>304</v>
       </c>
       <c r="D928" t="s">
-        <v>2643</v>
+        <v>305</v>
       </c>
     </row>
     <row r="929">
@@ -21304,13 +21322,13 @@
         <v>1733</v>
       </c>
       <c r="B929" t="s">
-        <v>2644</v>
+        <v>2645</v>
       </c>
       <c r="C929" t="s">
-        <v>2645</v>
+        <v>2646</v>
       </c>
       <c r="D929" t="s">
-        <v>2646</v>
+        <v>1885</v>
       </c>
     </row>
     <row r="930">
@@ -21461,10 +21479,10 @@
         <v>2677</v>
       </c>
       <c r="C940" t="s">
-        <v>2651</v>
+        <v>2678</v>
       </c>
       <c r="D940" t="s">
-        <v>2652</v>
+        <v>2679</v>
       </c>
     </row>
     <row r="941">
@@ -21472,13 +21490,13 @@
         <v>1733</v>
       </c>
       <c r="B941" t="s">
-        <v>2678</v>
+        <v>2680</v>
       </c>
       <c r="C941" t="s">
-        <v>2679</v>
+        <v>2681</v>
       </c>
       <c r="D941" t="s">
-        <v>2680</v>
+        <v>2682</v>
       </c>
     </row>
     <row r="942">
@@ -21486,13 +21504,13 @@
         <v>1733</v>
       </c>
       <c r="B942" t="s">
-        <v>2681</v>
+        <v>2683</v>
       </c>
       <c r="C942" t="s">
-        <v>2682</v>
+        <v>2657</v>
       </c>
       <c r="D942" t="s">
-        <v>2683</v>
+        <v>2658</v>
       </c>
     </row>
     <row r="943">
@@ -21587,10 +21605,10 @@
         <v>2702</v>
       </c>
       <c r="C949" t="s">
-        <v>2642</v>
+        <v>2703</v>
       </c>
       <c r="D949" t="s">
-        <v>2643</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="950">
@@ -21598,13 +21616,13 @@
         <v>1733</v>
       </c>
       <c r="B950" t="s">
-        <v>2703</v>
+        <v>2705</v>
       </c>
       <c r="C950" t="s">
-        <v>2704</v>
+        <v>2706</v>
       </c>
       <c r="D950" t="s">
-        <v>2705</v>
+        <v>2707</v>
       </c>
     </row>
     <row r="951">
@@ -21612,13 +21630,13 @@
         <v>1733</v>
       </c>
       <c r="B951" t="s">
-        <v>2706</v>
+        <v>2708</v>
       </c>
       <c r="C951" t="s">
-        <v>2707</v>
+        <v>2648</v>
       </c>
       <c r="D951" t="s">
-        <v>2708</v>
+        <v>2649</v>
       </c>
     </row>
     <row r="952">
@@ -21727,10 +21745,10 @@
         <v>2730</v>
       </c>
       <c r="C959" t="s">
-        <v>1282</v>
+        <v>2731</v>
       </c>
       <c r="D959" t="s">
-        <v>1283</v>
+        <v>2732</v>
       </c>
     </row>
     <row r="960">
@@ -21738,13 +21756,13 @@
         <v>1733</v>
       </c>
       <c r="B960" t="s">
-        <v>2731</v>
+        <v>2733</v>
       </c>
       <c r="C960" t="s">
-        <v>2732</v>
+        <v>2734</v>
       </c>
       <c r="D960" t="s">
-        <v>2733</v>
+        <v>2735</v>
       </c>
     </row>
     <row r="961">
@@ -21752,13 +21770,13 @@
         <v>1733</v>
       </c>
       <c r="B961" t="s">
-        <v>2734</v>
+        <v>2736</v>
       </c>
       <c r="C961" t="s">
-        <v>2735</v>
+        <v>1282</v>
       </c>
       <c r="D961" t="s">
-        <v>2736</v>
+        <v>1283</v>
       </c>
     </row>
     <row r="962">
@@ -21789,6 +21807,34 @@
         <v>2742</v>
       </c>
     </row>
+    <row r="964">
+      <c r="A964" t="s">
+        <v>1733</v>
+      </c>
+      <c r="B964" t="s">
+        <v>2743</v>
+      </c>
+      <c r="C964" t="s">
+        <v>2744</v>
+      </c>
+      <c r="D964" t="s">
+        <v>2745</v>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" t="s">
+        <v>1733</v>
+      </c>
+      <c r="B965" t="s">
+        <v>2746</v>
+      </c>
+      <c r="C965" t="s">
+        <v>2747</v>
+      </c>
+      <c r="D965" t="s">
+        <v>2748</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Staff access: a Manage access button on every row
</commit_message>
<xml_diff>
--- a/docs/amharic-review.xlsx
+++ b/docs/amharic-review.xlsx
@@ -8801,6 +8801,15 @@
   </si>
   <si>
     <t>users.active</t>
+  </si>
+  <si>
+    <t>users.manage</t>
+  </si>
+  <si>
+    <t>Manage access</t>
+  </si>
+  <si>
+    <t>መዳረሻ አስተዳድር</t>
   </si>
   <si>
     <t>users.roles</t>
@@ -23722,35 +23731,35 @@
         <v>2932</v>
       </c>
       <c r="C1034" t="s">
-        <v>1513</v>
+        <v>2933</v>
       </c>
       <c r="D1034" t="s">
-        <v>1514</v>
+        <v>2934</v>
       </c>
     </row>
     <row r="1035">
       <c r="A1035" t="s">
-        <v>2933</v>
+        <v>2038</v>
       </c>
       <c r="B1035" t="s">
-        <v>2934</v>
+        <v>2935</v>
       </c>
       <c r="C1035" t="s">
-        <v>2933</v>
+        <v>1513</v>
       </c>
       <c r="D1035" t="s">
-        <v>2935</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="1036">
       <c r="A1036" t="s">
-        <v>2933</v>
+        <v>2936</v>
       </c>
       <c r="B1036" t="s">
+        <v>2937</v>
+      </c>
+      <c r="C1036" t="s">
         <v>2936</v>
-      </c>
-      <c r="C1036" t="s">
-        <v>2937</v>
       </c>
       <c r="D1036" t="s">
         <v>2938</v>
@@ -23758,7 +23767,7 @@
     </row>
     <row r="1037">
       <c r="A1037" t="s">
-        <v>2933</v>
+        <v>2936</v>
       </c>
       <c r="B1037" t="s">
         <v>2939</v>
@@ -23772,7 +23781,7 @@
     </row>
     <row r="1038">
       <c r="A1038" t="s">
-        <v>2933</v>
+        <v>2936</v>
       </c>
       <c r="B1038" t="s">
         <v>2942</v>
@@ -23786,7 +23795,7 @@
     </row>
     <row r="1039">
       <c r="A1039" t="s">
-        <v>2041</v>
+        <v>2936</v>
       </c>
       <c r="B1039" t="s">
         <v>2945</v>
@@ -23834,10 +23843,10 @@
         <v>2954</v>
       </c>
       <c r="C1042" t="s">
-        <v>310</v>
+        <v>2955</v>
       </c>
       <c r="D1042" t="s">
-        <v>311</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="1043">
@@ -23845,13 +23854,13 @@
         <v>2041</v>
       </c>
       <c r="B1043" t="s">
-        <v>2955</v>
+        <v>2957</v>
       </c>
       <c r="C1043" t="s">
-        <v>2956</v>
+        <v>310</v>
       </c>
       <c r="D1043" t="s">
-        <v>2193</v>
+        <v>311</v>
       </c>
     </row>
     <row r="1044">
@@ -23859,13 +23868,13 @@
         <v>2041</v>
       </c>
       <c r="B1044" t="s">
-        <v>2957</v>
+        <v>2958</v>
       </c>
       <c r="C1044" t="s">
-        <v>2958</v>
+        <v>2959</v>
       </c>
       <c r="D1044" t="s">
-        <v>2959</v>
+        <v>2193</v>
       </c>
     </row>
     <row r="1045">
@@ -23974,10 +23983,10 @@
         <v>2981</v>
       </c>
       <c r="C1052" t="s">
-        <v>993</v>
+        <v>2982</v>
       </c>
       <c r="D1052" t="s">
-        <v>2982</v>
+        <v>2983</v>
       </c>
     </row>
     <row r="1053">
@@ -23985,10 +23994,10 @@
         <v>2041</v>
       </c>
       <c r="B1053" t="s">
-        <v>2983</v>
+        <v>2984</v>
       </c>
       <c r="C1053" t="s">
-        <v>2984</v>
+        <v>993</v>
       </c>
       <c r="D1053" t="s">
         <v>2985</v>
@@ -24030,10 +24039,10 @@
         <v>2992</v>
       </c>
       <c r="C1056" t="s">
-        <v>2967</v>
+        <v>2993</v>
       </c>
       <c r="D1056" t="s">
-        <v>2968</v>
+        <v>2994</v>
       </c>
     </row>
     <row r="1057">
@@ -24041,13 +24050,13 @@
         <v>2041</v>
       </c>
       <c r="B1057" t="s">
-        <v>2993</v>
+        <v>2995</v>
       </c>
       <c r="C1057" t="s">
-        <v>2994</v>
+        <v>2970</v>
       </c>
       <c r="D1057" t="s">
-        <v>2995</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="1058">
@@ -24156,10 +24165,10 @@
         <v>3017</v>
       </c>
       <c r="C1065" t="s">
-        <v>2958</v>
+        <v>3018</v>
       </c>
       <c r="D1065" t="s">
-        <v>2959</v>
+        <v>3019</v>
       </c>
     </row>
     <row r="1066">
@@ -24167,13 +24176,13 @@
         <v>2041</v>
       </c>
       <c r="B1066" t="s">
-        <v>3018</v>
+        <v>3020</v>
       </c>
       <c r="C1066" t="s">
-        <v>3019</v>
+        <v>2961</v>
       </c>
       <c r="D1066" t="s">
-        <v>3020</v>
+        <v>2962</v>
       </c>
     </row>
     <row r="1067">
@@ -24296,10 +24305,10 @@
         <v>3045</v>
       </c>
       <c r="C1075" t="s">
-        <v>1415</v>
+        <v>3046</v>
       </c>
       <c r="D1075" t="s">
-        <v>1416</v>
+        <v>3047</v>
       </c>
     </row>
     <row r="1076">
@@ -24307,13 +24316,13 @@
         <v>2041</v>
       </c>
       <c r="B1076" t="s">
-        <v>3046</v>
+        <v>3048</v>
       </c>
       <c r="C1076" t="s">
-        <v>3047</v>
+        <v>1415</v>
       </c>
       <c r="D1076" t="s">
-        <v>3048</v>
+        <v>1416</v>
       </c>
     </row>
     <row r="1077">
@@ -24358,6 +24367,20 @@
         <v>3057</v>
       </c>
     </row>
+    <row r="1080">
+      <c r="A1080" t="s">
+        <v>2041</v>
+      </c>
+      <c r="B1080" t="s">
+        <v>3058</v>
+      </c>
+      <c r="C1080" t="s">
+        <v>3059</v>
+      </c>
+      <c r="D1080" t="s">
+        <v>3060</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fixes from the browser pass: company name in setup card, contract and sample SMS; demo figure only for the original company; units chart; platform-only admins go to the console; clearer SMS gateway cards; company name on phones
</commit_message>
<xml_diff>
--- a/docs/amharic-review.xlsx
+++ b/docs/amharic-review.xlsx
@@ -8242,10 +8242,10 @@
     <t>contract.draft</t>
   </si>
   <si>
-    <t>Draft template. Dire Mall's lawyer should check the wording against Proclamation No. 1320/2024 before it is signed.</t>
-  </si>
-  <si>
-    <t>ረቂቅ ቅጽ። ከመፈረሙ በፊት የድሬ ሞል ጠበቃ ጽሑፉን ከአዋጅ ቁጥር 1320/2024 ጋር ማመሳከር አለበት።</t>
+    <t>Draft template. A lawyer should check the wording against Proclamation No. 1320/2024 before it is signed.</t>
+  </si>
+  <si>
+    <t>ረቂቅ ቅጽ። ከመፈረሙ በፊት ጠበቃ ጽሑፉን ከአዋጅ ቁጥር 1320/2024 ጋር ማመሳከር አለበት።</t>
   </si>
   <si>
     <t>contract.title</t>
@@ -10036,10 +10036,10 @@
     <t>first.title</t>
   </si>
   <si>
-    <t>Set up Dire Mall</t>
-  </si>
-  <si>
-    <t>ድሬ ሞልን ያዘጋጁ</t>
+    <t>Set up {c}</t>
+  </si>
+  <si>
+    <t>{c}ን ያዘጋጁ</t>
   </si>
   <si>
     <t>pw.hide</t>
@@ -10324,6 +10324,15 @@
     <t>መተላለፊያው ተገናኝቷል። መልዕክቶች እንደ {s} ይላካሉ።</t>
   </si>
   <si>
+    <t>sms.gatewayTest</t>
+  </si>
+  <si>
+    <t>Gateway status and test message</t>
+  </si>
+  <si>
+    <t>የመተላለፊያ ሁኔታና የሙከራ መልዕክት</t>
+  </si>
+  <si>
     <t>sms.inAmharic</t>
   </si>
   <si>
@@ -10480,10 +10489,10 @@
     <t>sms.noGateway</t>
   </si>
   <si>
-    <t>No SMS gateway is connected yet. Reminders and receipts are prepared and listed here, but they stay queued and nothing is sent until the gateway details are added (see the README, SMS).</t>
-  </si>
-  <si>
-    <t>እስካሁን የSMS መተላለፊያ አልተገናኘም። ማስታወሻዎችና ደረሰኞች ተዘጋጅተው እዚህ ይዘረዘራሉ፣ ነገር ግን የመተላለፊያው ዝርዝር እስኪጨመር ድረስ በወረፋ ይቆያሉ፤ ምንም አይላክም።</t>
+    <t>No SMS gateway is connected yet. Reminders and receipts are prepared and listed here, but they stay queued and nothing is sent until the gateway details are added Add your gateway in the box above.</t>
+  </si>
+  <si>
+    <t>እስካሁን የSMS መተላለፊያ አልተገናኘም። ማስታወሻዎችና ደረሰኞች ተዘጋጅተው እዚህ ይዘረዘራሉ፣ ነገር ግን የመተላለፊያው ዝርዝር እስኪጨመር ድረስ በወረፋ ይቆያሉ፤ ምንም አይላክም። መተላለፊያዎን ከላይ ባለው ሳጥን ውስጥ ያክሉ።</t>
   </si>
   <si>
     <t>sms.optIssued</t>
@@ -28596,10 +28605,10 @@
         <v>3454</v>
       </c>
       <c r="C1221" t="s">
-        <v>1832</v>
+        <v>3455</v>
       </c>
       <c r="D1221" t="s">
-        <v>3455</v>
+        <v>3456</v>
       </c>
     </row>
     <row r="1222">
@@ -28607,10 +28616,10 @@
         <v>2771</v>
       </c>
       <c r="B1222" t="s">
-        <v>3456</v>
+        <v>3457</v>
       </c>
       <c r="C1222" t="s">
-        <v>3457</v>
+        <v>1832</v>
       </c>
       <c r="D1222" t="s">
         <v>3458</v>
@@ -28624,10 +28633,10 @@
         <v>3459</v>
       </c>
       <c r="C1223" t="s">
-        <v>1429</v>
+        <v>3460</v>
       </c>
       <c r="D1223" t="s">
-        <v>3251</v>
+        <v>3461</v>
       </c>
     </row>
     <row r="1224">
@@ -28635,13 +28644,13 @@
         <v>2771</v>
       </c>
       <c r="B1224" t="s">
-        <v>3460</v>
+        <v>3462</v>
       </c>
       <c r="C1224" t="s">
-        <v>3461</v>
+        <v>1429</v>
       </c>
       <c r="D1224" t="s">
-        <v>3462</v>
+        <v>3251</v>
       </c>
     </row>
     <row r="1225">
@@ -28890,10 +28899,10 @@
         <v>3514</v>
       </c>
       <c r="C1242" t="s">
-        <v>336</v>
+        <v>3515</v>
       </c>
       <c r="D1242" t="s">
-        <v>337</v>
+        <v>3516</v>
       </c>
     </row>
     <row r="1243">
@@ -28901,13 +28910,13 @@
         <v>2771</v>
       </c>
       <c r="B1243" t="s">
-        <v>3515</v>
+        <v>3517</v>
       </c>
       <c r="C1243" t="s">
-        <v>3516</v>
+        <v>336</v>
       </c>
       <c r="D1243" t="s">
-        <v>3517</v>
+        <v>337</v>
       </c>
     </row>
     <row r="1244">
@@ -28918,10 +28927,10 @@
         <v>3518</v>
       </c>
       <c r="C1244" t="s">
-        <v>1767</v>
+        <v>3519</v>
       </c>
       <c r="D1244" t="s">
-        <v>1768</v>
+        <v>3520</v>
       </c>
     </row>
     <row r="1245">
@@ -28929,13 +28938,13 @@
         <v>2771</v>
       </c>
       <c r="B1245" t="s">
-        <v>3519</v>
+        <v>3521</v>
       </c>
       <c r="C1245" t="s">
-        <v>3520</v>
+        <v>1767</v>
       </c>
       <c r="D1245" t="s">
-        <v>3521</v>
+        <v>1768</v>
       </c>
     </row>
     <row r="1246">
@@ -28960,10 +28969,10 @@
         <v>3525</v>
       </c>
       <c r="C1247" t="s">
-        <v>566</v>
+        <v>3526</v>
       </c>
       <c r="D1247" t="s">
-        <v>567</v>
+        <v>3527</v>
       </c>
     </row>
     <row r="1248">
@@ -28971,13 +28980,13 @@
         <v>2771</v>
       </c>
       <c r="B1248" t="s">
-        <v>3526</v>
+        <v>3528</v>
       </c>
       <c r="C1248" t="s">
-        <v>3527</v>
+        <v>566</v>
       </c>
       <c r="D1248" t="s">
-        <v>3528</v>
+        <v>567</v>
       </c>
     </row>
     <row r="1249">
@@ -29002,10 +29011,10 @@
         <v>3532</v>
       </c>
       <c r="C1250" t="s">
-        <v>1089</v>
+        <v>3533</v>
       </c>
       <c r="D1250" t="s">
-        <v>1090</v>
+        <v>3534</v>
       </c>
     </row>
     <row r="1251">
@@ -29013,13 +29022,13 @@
         <v>2771</v>
       </c>
       <c r="B1251" t="s">
-        <v>3533</v>
+        <v>3535</v>
       </c>
       <c r="C1251" t="s">
-        <v>3534</v>
+        <v>1089</v>
       </c>
       <c r="D1251" t="s">
-        <v>3535</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="1252">
@@ -29159,7 +29168,7 @@
         <v>3564</v>
       </c>
       <c r="D1261" t="s">
-        <v>1060</v>
+        <v>3565</v>
       </c>
     </row>
     <row r="1262">
@@ -29167,13 +29176,13 @@
         <v>2771</v>
       </c>
       <c r="B1262" t="s">
-        <v>3565</v>
+        <v>3566</v>
       </c>
       <c r="C1262" t="s">
-        <v>3566</v>
+        <v>3567</v>
       </c>
       <c r="D1262" t="s">
-        <v>3567</v>
+        <v>1060</v>
       </c>
     </row>
     <row r="1263">
@@ -29285,7 +29294,7 @@
         <v>3590</v>
       </c>
       <c r="D1270" t="s">
-        <v>172</v>
+        <v>3591</v>
       </c>
     </row>
     <row r="1271">
@@ -29293,13 +29302,13 @@
         <v>2771</v>
       </c>
       <c r="B1271" t="s">
-        <v>3591</v>
+        <v>3592</v>
       </c>
       <c r="C1271" t="s">
-        <v>3592</v>
+        <v>3593</v>
       </c>
       <c r="D1271" t="s">
-        <v>1851</v>
+        <v>172</v>
       </c>
     </row>
     <row r="1272">
@@ -29307,10 +29316,10 @@
         <v>2771</v>
       </c>
       <c r="B1272" t="s">
-        <v>3593</v>
+        <v>3594</v>
       </c>
       <c r="C1272" t="s">
-        <v>3594</v>
+        <v>3595</v>
       </c>
       <c r="D1272" t="s">
         <v>1851</v>
@@ -29321,13 +29330,13 @@
         <v>2771</v>
       </c>
       <c r="B1273" t="s">
-        <v>3595</v>
+        <v>3596</v>
       </c>
       <c r="C1273" t="s">
-        <v>3596</v>
+        <v>3597</v>
       </c>
       <c r="D1273" t="s">
-        <v>3597</v>
+        <v>1851</v>
       </c>
     </row>
     <row r="1274">
@@ -29534,10 +29543,10 @@
         <v>3640</v>
       </c>
       <c r="C1288" t="s">
-        <v>3440</v>
+        <v>3641</v>
       </c>
       <c r="D1288" t="s">
-        <v>3441</v>
+        <v>3642</v>
       </c>
     </row>
     <row r="1289">
@@ -29545,13 +29554,13 @@
         <v>2771</v>
       </c>
       <c r="B1289" t="s">
-        <v>3641</v>
+        <v>3643</v>
       </c>
       <c r="C1289" t="s">
-        <v>3642</v>
+        <v>3443</v>
       </c>
       <c r="D1289" t="s">
-        <v>3643</v>
+        <v>3444</v>
       </c>
     </row>
     <row r="1290">
@@ -29562,10 +29571,10 @@
         <v>3644</v>
       </c>
       <c r="C1290" t="s">
-        <v>3449</v>
+        <v>3645</v>
       </c>
       <c r="D1290" t="s">
-        <v>3450</v>
+        <v>3646</v>
       </c>
     </row>
     <row r="1291">
@@ -29573,13 +29582,13 @@
         <v>2771</v>
       </c>
       <c r="B1291" t="s">
-        <v>3645</v>
+        <v>3647</v>
       </c>
       <c r="C1291" t="s">
-        <v>3646</v>
+        <v>3452</v>
       </c>
       <c r="D1291" t="s">
-        <v>3647</v>
+        <v>3453</v>
       </c>
     </row>
     <row r="1292">
@@ -29590,10 +29599,10 @@
         <v>3648</v>
       </c>
       <c r="C1292" t="s">
-        <v>3452</v>
+        <v>3649</v>
       </c>
       <c r="D1292" t="s">
-        <v>3453</v>
+        <v>3650</v>
       </c>
     </row>
     <row r="1293">
@@ -29601,13 +29610,13 @@
         <v>2771</v>
       </c>
       <c r="B1293" t="s">
-        <v>3649</v>
+        <v>3651</v>
       </c>
       <c r="C1293" t="s">
-        <v>3650</v>
+        <v>3455</v>
       </c>
       <c r="D1293" t="s">
-        <v>3651</v>
+        <v>3456</v>
       </c>
     </row>
     <row r="1294">
@@ -29688,10 +29697,10 @@
         <v>3667</v>
       </c>
       <c r="C1299" t="s">
-        <v>3091</v>
+        <v>3668</v>
       </c>
       <c r="D1299" t="s">
-        <v>483</v>
+        <v>3669</v>
       </c>
     </row>
     <row r="1300">
@@ -29699,13 +29708,13 @@
         <v>2771</v>
       </c>
       <c r="B1300" t="s">
-        <v>3668</v>
+        <v>3670</v>
       </c>
       <c r="C1300" t="s">
-        <v>3669</v>
+        <v>3091</v>
       </c>
       <c r="D1300" t="s">
-        <v>3670</v>
+        <v>483</v>
       </c>
     </row>
     <row r="1301">
@@ -29738,16 +29747,16 @@
     </row>
     <row r="1303">
       <c r="A1303" t="s">
-        <v>2786</v>
+        <v>2771</v>
       </c>
       <c r="B1303" t="s">
         <v>3677</v>
       </c>
       <c r="C1303" t="s">
-        <v>1281</v>
+        <v>3678</v>
       </c>
       <c r="D1303" t="s">
-        <v>1282</v>
+        <v>3679</v>
       </c>
     </row>
     <row r="1304">
@@ -29755,13 +29764,13 @@
         <v>2786</v>
       </c>
       <c r="B1304" t="s">
-        <v>3678</v>
+        <v>3680</v>
       </c>
       <c r="C1304" t="s">
-        <v>3679</v>
+        <v>1281</v>
       </c>
       <c r="D1304" t="s">
-        <v>3680</v>
+        <v>1282</v>
       </c>
     </row>
     <row r="1305">
@@ -29786,35 +29795,35 @@
         <v>3684</v>
       </c>
       <c r="C1306" t="s">
-        <v>2164</v>
+        <v>3685</v>
       </c>
       <c r="D1306" t="s">
-        <v>2165</v>
+        <v>3686</v>
       </c>
     </row>
     <row r="1307">
       <c r="A1307" t="s">
-        <v>3685</v>
+        <v>2786</v>
       </c>
       <c r="B1307" t="s">
-        <v>3686</v>
+        <v>3687</v>
       </c>
       <c r="C1307" t="s">
-        <v>3685</v>
+        <v>2164</v>
       </c>
       <c r="D1307" t="s">
-        <v>3687</v>
+        <v>2165</v>
       </c>
     </row>
     <row r="1308">
       <c r="A1308" t="s">
-        <v>3685</v>
+        <v>3688</v>
       </c>
       <c r="B1308" t="s">
+        <v>3689</v>
+      </c>
+      <c r="C1308" t="s">
         <v>3688</v>
-      </c>
-      <c r="C1308" t="s">
-        <v>3689</v>
       </c>
       <c r="D1308" t="s">
         <v>3690</v>
@@ -29822,7 +29831,7 @@
     </row>
     <row r="1309">
       <c r="A1309" t="s">
-        <v>3685</v>
+        <v>3688</v>
       </c>
       <c r="B1309" t="s">
         <v>3691</v>
@@ -29836,7 +29845,7 @@
     </row>
     <row r="1310">
       <c r="A1310" t="s">
-        <v>3685</v>
+        <v>3688</v>
       </c>
       <c r="B1310" t="s">
         <v>3694</v>
@@ -29850,7 +29859,7 @@
     </row>
     <row r="1311">
       <c r="A1311" t="s">
-        <v>2789</v>
+        <v>3688</v>
       </c>
       <c r="B1311" t="s">
         <v>3697</v>
@@ -29898,10 +29907,10 @@
         <v>3706</v>
       </c>
       <c r="C1314" t="s">
-        <v>310</v>
+        <v>3707</v>
       </c>
       <c r="D1314" t="s">
-        <v>311</v>
+        <v>3708</v>
       </c>
     </row>
     <row r="1315">
@@ -29909,13 +29918,13 @@
         <v>2789</v>
       </c>
       <c r="B1315" t="s">
-        <v>3707</v>
+        <v>3709</v>
       </c>
       <c r="C1315" t="s">
-        <v>3708</v>
+        <v>310</v>
       </c>
       <c r="D1315" t="s">
-        <v>2941</v>
+        <v>311</v>
       </c>
     </row>
     <row r="1316">
@@ -29923,13 +29932,13 @@
         <v>2789</v>
       </c>
       <c r="B1316" t="s">
-        <v>3709</v>
+        <v>3710</v>
       </c>
       <c r="C1316" t="s">
-        <v>3710</v>
+        <v>3711</v>
       </c>
       <c r="D1316" t="s">
-        <v>3711</v>
+        <v>2941</v>
       </c>
     </row>
     <row r="1317">
@@ -30038,10 +30047,10 @@
         <v>3733</v>
       </c>
       <c r="C1324" t="s">
-        <v>1272</v>
+        <v>3734</v>
       </c>
       <c r="D1324" t="s">
-        <v>3734</v>
+        <v>3735</v>
       </c>
     </row>
     <row r="1325">
@@ -30049,10 +30058,10 @@
         <v>2789</v>
       </c>
       <c r="B1325" t="s">
-        <v>3735</v>
+        <v>3736</v>
       </c>
       <c r="C1325" t="s">
-        <v>3736</v>
+        <v>1272</v>
       </c>
       <c r="D1325" t="s">
         <v>3737</v>
@@ -30094,10 +30103,10 @@
         <v>3744</v>
       </c>
       <c r="C1328" t="s">
-        <v>3719</v>
+        <v>3745</v>
       </c>
       <c r="D1328" t="s">
-        <v>3720</v>
+        <v>3746</v>
       </c>
     </row>
     <row r="1329">
@@ -30105,13 +30114,13 @@
         <v>2789</v>
       </c>
       <c r="B1329" t="s">
-        <v>3745</v>
+        <v>3747</v>
       </c>
       <c r="C1329" t="s">
-        <v>3746</v>
+        <v>3722</v>
       </c>
       <c r="D1329" t="s">
-        <v>3747</v>
+        <v>3723</v>
       </c>
     </row>
     <row r="1330">
@@ -30220,10 +30229,10 @@
         <v>3769</v>
       </c>
       <c r="C1337" t="s">
-        <v>3710</v>
+        <v>3770</v>
       </c>
       <c r="D1337" t="s">
-        <v>3711</v>
+        <v>3771</v>
       </c>
     </row>
     <row r="1338">
@@ -30231,13 +30240,13 @@
         <v>2789</v>
       </c>
       <c r="B1338" t="s">
-        <v>3770</v>
+        <v>3772</v>
       </c>
       <c r="C1338" t="s">
-        <v>3771</v>
+        <v>3713</v>
       </c>
       <c r="D1338" t="s">
-        <v>3772</v>
+        <v>3714</v>
       </c>
     </row>
     <row r="1339">
@@ -30360,10 +30369,10 @@
         <v>3797</v>
       </c>
       <c r="C1347" t="s">
-        <v>1730</v>
+        <v>3798</v>
       </c>
       <c r="D1347" t="s">
-        <v>1845</v>
+        <v>3799</v>
       </c>
     </row>
     <row r="1348">
@@ -30371,13 +30380,13 @@
         <v>2789</v>
       </c>
       <c r="B1348" t="s">
-        <v>3798</v>
+        <v>3800</v>
       </c>
       <c r="C1348" t="s">
-        <v>3799</v>
+        <v>1730</v>
       </c>
       <c r="D1348" t="s">
-        <v>3800</v>
+        <v>1845</v>
       </c>
     </row>
     <row r="1349">
@@ -30422,6 +30431,20 @@
         <v>3809</v>
       </c>
     </row>
+    <row r="1352">
+      <c r="A1352" t="s">
+        <v>2789</v>
+      </c>
+      <c r="B1352" t="s">
+        <v>3810</v>
+      </c>
+      <c r="C1352" t="s">
+        <v>3811</v>
+      </c>
+      <c r="D1352" t="s">
+        <v>3812</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>